<commit_message>
Semana 1: Etapa 1 adaptada para secretarias (visão da rede)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AahsCeqM2DTecRKsTTfJbG
</commit_message>
<xml_diff>
--- a/kobo/gestores_semana1_diagnostico.xlsx
+++ b/kobo/gestores_semana1_diagnostico.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J127"/>
+  <dimension ref="A1:J157"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2170,26 +2170,26 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>select_one agua_fonte</t>
+          <t>begin_group</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>q1_5</t>
+          <t>e1_escola</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Q1.5. Fonte de abastecimento de água</t>
+          <t>Água, esgoto e resíduos — local</t>
         </is>
       </c>
       <c r="D64" t="inlineStr"/>
-      <c r="E64" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="F64" t="inlineStr"/>
+      <c r="E64" t="inlineStr"/>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>${q0_9}='escola'</t>
+        </is>
+      </c>
       <c r="G64" t="inlineStr"/>
       <c r="H64" t="inlineStr"/>
       <c r="I64" t="inlineStr"/>
@@ -2198,26 +2198,26 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>select_one agua_fonte</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>q1_5_outro</t>
+          <t>q1_5</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Especifique (Outro)</t>
+          <t>Q1.5. Fonte de abastecimento de água</t>
         </is>
       </c>
       <c r="D65" t="inlineStr"/>
-      <c r="E65" t="inlineStr"/>
-      <c r="F65" t="inlineStr">
-        <is>
-          <t>${q1_5}='outro'</t>
-        </is>
-      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr"/>
       <c r="G65" t="inlineStr"/>
       <c r="H65" t="inlineStr"/>
       <c r="I65" t="inlineStr"/>
@@ -2226,22 +2226,26 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>select_one sim_nao_ns</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>q1_6</t>
+          <t>q1_5_outro</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Q1.6. Há interrupções no abastecimento de água?</t>
+          <t>Especifique (Outro)</t>
         </is>
       </c>
       <c r="D66" t="inlineStr"/>
       <c r="E66" t="inlineStr"/>
-      <c r="F66" t="inlineStr"/>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>${q1_5}='outro'</t>
+        </is>
+      </c>
       <c r="G66" t="inlineStr"/>
       <c r="H66" t="inlineStr"/>
       <c r="I66" t="inlineStr"/>
@@ -2250,31 +2254,23 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>select_one sim_nao_ns</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>q1_7</t>
+          <t>q1_6</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Q1.7. Em que período(s) isso costuma ocorrer?</t>
+          <t>Q1.6. Há interrupções no abastecimento de água?</t>
         </is>
       </c>
       <c r="D67" t="inlineStr"/>
       <c r="E67" t="inlineStr"/>
-      <c r="F67" t="inlineStr">
-        <is>
-          <t>${q1_6}='sim'</t>
-        </is>
-      </c>
-      <c r="G67" t="inlineStr">
-        <is>
-          <t>multiline</t>
-        </is>
-      </c>
+      <c r="F67" t="inlineStr"/>
+      <c r="G67" t="inlineStr"/>
       <c r="H67" t="inlineStr"/>
       <c r="I67" t="inlineStr"/>
       <c r="J67" t="inlineStr"/>
@@ -2282,23 +2278,31 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>select_one sim_nao_ns</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>q1_8</t>
+          <t>q1_7</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Q1.8. Existe monitoramento da qualidade da água?</t>
+          <t>Q1.7. Em que período(s) isso costuma ocorrer?</t>
         </is>
       </c>
       <c r="D68" t="inlineStr"/>
       <c r="E68" t="inlineStr"/>
-      <c r="F68" t="inlineStr"/>
-      <c r="G68" t="inlineStr"/>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>${q1_6}='sim'</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>multiline</t>
+        </is>
+      </c>
       <c r="H68" t="inlineStr"/>
       <c r="I68" t="inlineStr"/>
       <c r="J68" t="inlineStr"/>
@@ -2306,31 +2310,23 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>select_one sim_nao_ns</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>q1_9</t>
+          <t>q1_8</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Q1.9. Quem é responsável por esse monitoramento?</t>
+          <t>Q1.8. Existe monitoramento da qualidade da água?</t>
         </is>
       </c>
       <c r="D69" t="inlineStr"/>
       <c r="E69" t="inlineStr"/>
-      <c r="F69" t="inlineStr">
-        <is>
-          <t>${q1_8}='sim'</t>
-        </is>
-      </c>
-      <c r="G69" t="inlineStr">
-        <is>
-          <t>multiline</t>
-        </is>
-      </c>
+      <c r="F69" t="inlineStr"/>
+      <c r="G69" t="inlineStr"/>
       <c r="H69" t="inlineStr"/>
       <c r="I69" t="inlineStr"/>
       <c r="J69" t="inlineStr"/>
@@ -2338,17 +2334,17 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>select_one sim_nao_ns</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>q1_10</t>
+          <t>q1_9</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Q1.10. Existem registros desse monitoramento?</t>
+          <t>Q1.9. Quem é responsável por esse monitoramento?</t>
         </is>
       </c>
       <c r="D70" t="inlineStr"/>
@@ -2358,7 +2354,11 @@
           <t>${q1_8}='sim'</t>
         </is>
       </c>
-      <c r="G70" t="inlineStr"/>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>multiline</t>
+        </is>
+      </c>
       <c r="H70" t="inlineStr"/>
       <c r="I70" t="inlineStr"/>
       <c r="J70" t="inlineStr"/>
@@ -2366,22 +2366,26 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>select_multiple infra_hidrica</t>
+          <t>select_one sim_nao_ns</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>q1_11</t>
+          <t>q1_10</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Q1.11. Infraestrutura hídrica disponível</t>
+          <t>Q1.10. Existem registros desse monitoramento?</t>
         </is>
       </c>
       <c r="D71" t="inlineStr"/>
       <c r="E71" t="inlineStr"/>
-      <c r="F71" t="inlineStr"/>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>${q1_8}='sim'</t>
+        </is>
+      </c>
       <c r="G71" t="inlineStr"/>
       <c r="H71" t="inlineStr"/>
       <c r="I71" t="inlineStr"/>
@@ -2390,26 +2394,22 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>select_multiple infra_hidrica</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>q1_11_outro</t>
+          <t>q1_11</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Especifique (Outro)</t>
+          <t>Q1.11. Infraestrutura hídrica disponível</t>
         </is>
       </c>
       <c r="D72" t="inlineStr"/>
       <c r="E72" t="inlineStr"/>
-      <c r="F72" t="inlineStr">
-        <is>
-          <t>selected(${q1_11}, 'outro')</t>
-        </is>
-      </c>
+      <c r="F72" t="inlineStr"/>
       <c r="G72" t="inlineStr"/>
       <c r="H72" t="inlineStr"/>
       <c r="I72" t="inlineStr"/>
@@ -2418,22 +2418,26 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>select_multiple esgoto</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>q1_12</t>
+          <t>q1_11_outro</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Q1.12. Destinação do esgoto</t>
+          <t>Especifique (Outro)</t>
         </is>
       </c>
       <c r="D73" t="inlineStr"/>
       <c r="E73" t="inlineStr"/>
-      <c r="F73" t="inlineStr"/>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>selected(${q1_11}, 'outro')</t>
+        </is>
+      </c>
       <c r="G73" t="inlineStr"/>
       <c r="H73" t="inlineStr"/>
       <c r="I73" t="inlineStr"/>
@@ -2442,26 +2446,22 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>select_multiple esgoto</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>q1_12_outro</t>
+          <t>q1_12</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Especifique (Outro)</t>
+          <t>Q1.12. Destinação do esgoto</t>
         </is>
       </c>
       <c r="D74" t="inlineStr"/>
       <c r="E74" t="inlineStr"/>
-      <c r="F74" t="inlineStr">
-        <is>
-          <t>selected(${q1_12}, 'outro')</t>
-        </is>
-      </c>
+      <c r="F74" t="inlineStr"/>
       <c r="G74" t="inlineStr"/>
       <c r="H74" t="inlineStr"/>
       <c r="I74" t="inlineStr"/>
@@ -2470,22 +2470,26 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>select_one sim_nao_ns</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>q1_13</t>
+          <t>q1_12_outro</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Q1.13. Há esgoto a céu aberto no entorno do local?</t>
+          <t>Especifique (Outro)</t>
         </is>
       </c>
       <c r="D75" t="inlineStr"/>
       <c r="E75" t="inlineStr"/>
-      <c r="F75" t="inlineStr"/>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>selected(${q1_12}, 'outro')</t>
+        </is>
+      </c>
       <c r="G75" t="inlineStr"/>
       <c r="H75" t="inlineStr"/>
       <c r="I75" t="inlineStr"/>
@@ -2499,20 +2503,16 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>q1_14</t>
+          <t>q1_13</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Q1.14. Ocorrem alagamentos neste local ou no entorno?</t>
+          <t>Q1.13. Há esgoto a céu aberto no entorno do local?</t>
         </is>
       </c>
       <c r="D76" t="inlineStr"/>
-      <c r="E76" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
+      <c r="E76" t="inlineStr"/>
       <c r="F76" t="inlineStr"/>
       <c r="G76" t="inlineStr"/>
       <c r="H76" t="inlineStr"/>
@@ -2522,31 +2522,27 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>select_one sim_nao_ns</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>q1_15</t>
+          <t>q1_14</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Q1.15. Onde costumam ocorrer?</t>
+          <t>Q1.14. Ocorrem alagamentos neste local ou no entorno?</t>
         </is>
       </c>
       <c r="D77" t="inlineStr"/>
-      <c r="E77" t="inlineStr"/>
-      <c r="F77" t="inlineStr">
-        <is>
-          <t>${q1_14}='sim'</t>
-        </is>
-      </c>
-      <c r="G77" t="inlineStr">
-        <is>
-          <t>multiline</t>
-        </is>
-      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr"/>
+      <c r="G77" t="inlineStr"/>
       <c r="H77" t="inlineStr"/>
       <c r="I77" t="inlineStr"/>
       <c r="J77" t="inlineStr"/>
@@ -2554,17 +2550,17 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>select_multiple impacto_alag</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>q1_16</t>
+          <t>q1_15</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Q1.16. Impactos observados nesses episódios</t>
+          <t>Q1.15. Onde costumam ocorrer?</t>
         </is>
       </c>
       <c r="D78" t="inlineStr"/>
@@ -2574,7 +2570,11 @@
           <t>${q1_14}='sim'</t>
         </is>
       </c>
-      <c r="G78" t="inlineStr"/>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>multiline</t>
+        </is>
+      </c>
       <c r="H78" t="inlineStr"/>
       <c r="I78" t="inlineStr"/>
       <c r="J78" t="inlineStr"/>
@@ -2582,24 +2582,24 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>select_multiple impacto_alag</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>q1_16_outro</t>
+          <t>q1_16</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Especifique (Outro)</t>
+          <t>Q1.16. Impactos observados nesses episódios</t>
         </is>
       </c>
       <c r="D79" t="inlineStr"/>
       <c r="E79" t="inlineStr"/>
       <c r="F79" t="inlineStr">
         <is>
-          <t>(${q1_14}='sim') and selected(${q1_16}, 'outro')</t>
+          <t>${q1_14}='sim'</t>
         </is>
       </c>
       <c r="G79" t="inlineStr"/>
@@ -2610,22 +2610,26 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>select_one sim_nao_ns</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>q1_17</t>
+          <t>q1_16_outro</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Q1.17. Há separação de resíduos neste local?</t>
+          <t>Especifique (Outro)</t>
         </is>
       </c>
       <c r="D80" t="inlineStr"/>
       <c r="E80" t="inlineStr"/>
-      <c r="F80" t="inlineStr"/>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>(${q1_14}='sim') and selected(${q1_16}, 'outro')</t>
+        </is>
+      </c>
       <c r="G80" t="inlineStr"/>
       <c r="H80" t="inlineStr"/>
       <c r="I80" t="inlineStr"/>
@@ -2634,17 +2638,17 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>select_multiple destino_res</t>
+          <t>select_one sim_nao_ns</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>q1_18</t>
+          <t>q1_17</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Q1.18. Destinação dos resíduos</t>
+          <t>Q1.17. Há separação de resíduos neste local?</t>
         </is>
       </c>
       <c r="D81" t="inlineStr"/>
@@ -2658,26 +2662,22 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>select_multiple destino_res</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>q1_18_outro</t>
+          <t>q1_18</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Especifique (Outro)</t>
+          <t>Q1.18. Destinação dos resíduos</t>
         </is>
       </c>
       <c r="D82" t="inlineStr"/>
       <c r="E82" t="inlineStr"/>
-      <c r="F82" t="inlineStr">
-        <is>
-          <t>selected(${q1_18}, 'outro')</t>
-        </is>
-      </c>
+      <c r="F82" t="inlineStr"/>
       <c r="G82" t="inlineStr"/>
       <c r="H82" t="inlineStr"/>
       <c r="I82" t="inlineStr"/>
@@ -2686,65 +2686,65 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>select_multiple prob_res</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>q1_19</t>
+          <t>q1_18_outro</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Q1.19. Existem problemas relacionados a resíduos no entorno do local?</t>
-        </is>
-      </c>
-      <c r="D83" t="inlineStr">
-        <is>
-          <t>Considere a área imediatamente ao redor do local, não o município inteiro.</t>
-        </is>
-      </c>
+          <t>Especifique (Outro)</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr"/>
       <c r="E83" t="inlineStr"/>
-      <c r="F83" t="inlineStr"/>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>selected(${q1_18}, 'outro')</t>
+        </is>
+      </c>
       <c r="G83" t="inlineStr"/>
-      <c r="H83" t="inlineStr">
-        <is>
-          <t>not((selected(., 'nenhum') or selected(., 'nao_sabe')) and count-selected(.) &gt; 1)</t>
-        </is>
-      </c>
-      <c r="I83" t="inlineStr">
-        <is>
-          <t>"Nenhum" e "Não sabe" não podem ser combinados com outras opções.</t>
-        </is>
-      </c>
+      <c r="H83" t="inlineStr"/>
+      <c r="I83" t="inlineStr"/>
       <c r="J83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>select_multiple prob_res</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>q1_19_outro</t>
+          <t>q1_19</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Especifique (Outro)</t>
-        </is>
-      </c>
-      <c r="D84" t="inlineStr"/>
+          <t>Q1.19. Existem problemas relacionados a resíduos no entorno do local?</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>Considere a área imediatamente ao redor do local, não o município inteiro.</t>
+        </is>
+      </c>
       <c r="E84" t="inlineStr"/>
-      <c r="F84" t="inlineStr">
-        <is>
-          <t>selected(${q1_19}, 'outro')</t>
-        </is>
-      </c>
+      <c r="F84" t="inlineStr"/>
       <c r="G84" t="inlineStr"/>
-      <c r="H84" t="inlineStr"/>
-      <c r="I84" t="inlineStr"/>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>not((selected(., 'nenhum') or selected(., 'nao_sabe')) and count-selected(.) &gt; 1)</t>
+        </is>
+      </c>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>"Nenhum" e "Não sabe" não podem ser combinados com outras opções.</t>
+        </is>
+      </c>
       <c r="J84" t="inlineStr"/>
     </row>
     <row r="85">
@@ -2755,26 +2755,22 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>q1_20</t>
+          <t>q1_19_outro</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Q1.20. Descreva esses problemas</t>
+          <t>Especifique (Outro)</t>
         </is>
       </c>
       <c r="D85" t="inlineStr"/>
       <c r="E85" t="inlineStr"/>
       <c r="F85" t="inlineStr">
         <is>
-          <t>${q1_19} != '' and not(selected(${q1_19}, 'nenhum')) and not(selected(${q1_19}, 'nao_sabe'))</t>
-        </is>
-      </c>
-      <c r="G85" t="inlineStr">
-        <is>
-          <t>multiline</t>
-        </is>
-      </c>
+          <t>selected(${q1_19}, 'outro')</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr"/>
       <c r="H85" t="inlineStr"/>
       <c r="I85" t="inlineStr"/>
       <c r="J85" t="inlineStr"/>
@@ -2782,31 +2778,31 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>select_multiple elementos</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>q1_21</t>
+          <t>q1_20</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Q1.21. Elementos presentes no território ao redor do local</t>
-        </is>
-      </c>
-      <c r="D86" t="inlineStr">
-        <is>
-          <t>Considere o território mais imediato do local — em geral o bairro ou a região do entorno em que a comunidade escolar circula, não o município inteiro. A existência de um elemento não significa, por si só, risco ou impacto — isso será explorado a seguir.</t>
-        </is>
-      </c>
-      <c r="E86" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="F86" t="inlineStr"/>
-      <c r="G86" t="inlineStr"/>
+          <t>Q1.20. Descreva esses problemas</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr"/>
+      <c r="E86" t="inlineStr"/>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>${q1_19} != '' and not(selected(${q1_19}, 'nenhum')) and not(selected(${q1_19}, 'nao_sabe'))</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>multiline</t>
+        </is>
+      </c>
       <c r="H86" t="inlineStr"/>
       <c r="I86" t="inlineStr"/>
       <c r="J86" t="inlineStr"/>
@@ -2814,26 +2810,14 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="B87" t="inlineStr">
-        <is>
-          <t>q1_21_outro</t>
-        </is>
-      </c>
-      <c r="C87" t="inlineStr">
-        <is>
-          <t>Especifique (Outro)</t>
-        </is>
-      </c>
+          <t>end_group</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr"/>
+      <c r="C87" t="inlineStr"/>
       <c r="D87" t="inlineStr"/>
       <c r="E87" t="inlineStr"/>
-      <c r="F87" t="inlineStr">
-        <is>
-          <t>selected(${q1_21}, 'outro')</t>
-        </is>
-      </c>
+      <c r="F87" t="inlineStr"/>
       <c r="G87" t="inlineStr"/>
       <c r="H87" t="inlineStr"/>
       <c r="I87" t="inlineStr"/>
@@ -2847,26 +2831,22 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>t1_22</t>
+          <t>e1_rede</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Q1.22. Para cada elemento selecionado, qual sua relação com o local/comunidade?</t>
+          <t>Água, esgoto e resíduos — escolas da rede</t>
         </is>
       </c>
       <c r="D88" t="inlineStr"/>
       <c r="E88" t="inlineStr"/>
       <c r="F88" t="inlineStr">
         <is>
-          <t>${q1_21} != ''</t>
-        </is>
-      </c>
-      <c r="G88" t="inlineStr">
-        <is>
-          <t>table-list</t>
-        </is>
-      </c>
+          <t>${q0_9} != 'escola'</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr"/>
       <c r="H88" t="inlineStr"/>
       <c r="I88" t="inlineStr"/>
       <c r="J88" t="inlineStr"/>
@@ -2874,26 +2854,22 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>select_multiple relacao_elem</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>q1_22_01</t>
+          <t>e1_rede_nota</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Rios/córregos</t>
+          <t>Responda com base na sua visão geral das locais da rede/região de atuação. Estimativas são bem-vindas; "Não sabe" é uma resposta válida e vira lacuna de conhecimento registrada.</t>
         </is>
       </c>
       <c r="D89" t="inlineStr"/>
       <c r="E89" t="inlineStr"/>
-      <c r="F89" t="inlineStr">
-        <is>
-          <t>selected(${q1_21}, 'rios_corregos')</t>
-        </is>
-      </c>
+      <c r="F89" t="inlineStr"/>
       <c r="G89" t="inlineStr"/>
       <c r="H89" t="inlineStr"/>
       <c r="I89" t="inlineStr"/>
@@ -2902,26 +2878,26 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>select_multiple relacao_elem</t>
+          <t>select_multiple termica</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>q1_22_02</t>
+          <t>q1_3r</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Lagoas/lagos/reservatórios</t>
-        </is>
-      </c>
-      <c r="D90" t="inlineStr"/>
+          <t>Q1.3. Condição térmica das salas de aula nas escolas da rede</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>Marque todas as situações que se aplicam à rede.</t>
+        </is>
+      </c>
       <c r="E90" t="inlineStr"/>
-      <c r="F90" t="inlineStr">
-        <is>
-          <t>selected(${q1_21}, 'lagoas_lagos_reservatorios')</t>
-        </is>
-      </c>
+      <c r="F90" t="inlineStr"/>
       <c r="G90" t="inlineStr"/>
       <c r="H90" t="inlineStr"/>
       <c r="I90" t="inlineStr"/>
@@ -2930,26 +2906,22 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>select_multiple relacao_elem</t>
+          <t>select_multiple prob_estrut</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>q1_22_03</t>
+          <t>q1_4r</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Vegetação</t>
+          <t>Q1.4. Problemas estruturais mais comuns nas escolas da rede</t>
         </is>
       </c>
       <c r="D91" t="inlineStr"/>
       <c r="E91" t="inlineStr"/>
-      <c r="F91" t="inlineStr">
-        <is>
-          <t>selected(${q1_21}, 'vegetacao')</t>
-        </is>
-      </c>
+      <c r="F91" t="inlineStr"/>
       <c r="G91" t="inlineStr"/>
       <c r="H91" t="inlineStr"/>
       <c r="I91" t="inlineStr"/>
@@ -2958,24 +2930,24 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>select_multiple relacao_elem</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>q1_22_04</t>
+          <t>q1_4r_outro</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Parques</t>
+          <t>Especifique (Outro)</t>
         </is>
       </c>
       <c r="D92" t="inlineStr"/>
       <c r="E92" t="inlineStr"/>
       <c r="F92" t="inlineStr">
         <is>
-          <t>selected(${q1_21}, 'parques')</t>
+          <t>selected(${q1_4r}, 'outro')</t>
         </is>
       </c>
       <c r="G92" t="inlineStr"/>
@@ -2986,26 +2958,26 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>select_multiple relacao_elem</t>
+          <t>select_multiple agua_fonte</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>q1_22_05</t>
+          <t>q1_5r</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Encostas</t>
+          <t>Q1.5. Fontes de abastecimento de água das escolas da rede</t>
         </is>
       </c>
       <c r="D93" t="inlineStr"/>
-      <c r="E93" t="inlineStr"/>
-      <c r="F93" t="inlineStr">
-        <is>
-          <t>selected(${q1_21}, 'encostas')</t>
-        </is>
-      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr"/>
       <c r="G93" t="inlineStr"/>
       <c r="H93" t="inlineStr"/>
       <c r="I93" t="inlineStr"/>
@@ -3014,24 +2986,24 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>select_multiple relacao_elem</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>q1_22_06</t>
+          <t>q1_5r_outro</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Agricultura</t>
+          <t>Especifique (Outro)</t>
         </is>
       </c>
       <c r="D94" t="inlineStr"/>
       <c r="E94" t="inlineStr"/>
       <c r="F94" t="inlineStr">
         <is>
-          <t>selected(${q1_21}, 'agricultura')</t>
+          <t>selected(${q1_5r}, 'outro')</t>
         </is>
       </c>
       <c r="G94" t="inlineStr"/>
@@ -3042,26 +3014,22 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>select_multiple relacao_elem</t>
+          <t>select_one qtd_rede</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>q1_22_07</t>
+          <t>q1_6r</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Indústria</t>
+          <t>Q1.6. Em quantas escolas da rede há interrupções no abastecimento de água?</t>
         </is>
       </c>
       <c r="D95" t="inlineStr"/>
       <c r="E95" t="inlineStr"/>
-      <c r="F95" t="inlineStr">
-        <is>
-          <t>selected(${q1_21}, 'industria')</t>
-        </is>
-      </c>
+      <c r="F95" t="inlineStr"/>
       <c r="G95" t="inlineStr"/>
       <c r="H95" t="inlineStr"/>
       <c r="I95" t="inlineStr"/>
@@ -3070,27 +3038,31 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>select_multiple relacao_elem</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>q1_22_08</t>
+          <t>q1_7r</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Mineração</t>
+          <t>Q1.7. Em que período(s) isso costuma ocorrer?</t>
         </is>
       </c>
       <c r="D96" t="inlineStr"/>
       <c r="E96" t="inlineStr"/>
       <c r="F96" t="inlineStr">
         <is>
-          <t>selected(${q1_21}, 'mineracao')</t>
-        </is>
-      </c>
-      <c r="G96" t="inlineStr"/>
+          <t>${q1_6r} != '' and ${q1_6r} != 'em_nenhuma' and ${q1_6r} != 'nao_sabe'</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>multiline</t>
+        </is>
+      </c>
       <c r="H96" t="inlineStr"/>
       <c r="I96" t="inlineStr"/>
       <c r="J96" t="inlineStr"/>
@@ -3098,26 +3070,22 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>select_multiple relacao_elem</t>
+          <t>select_one qtd_rede</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>q1_22_09</t>
+          <t>q1_8r</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Aterro/lixão</t>
+          <t>Q1.8. Em quantas escolas da rede há monitoramento da qualidade da água?</t>
         </is>
       </c>
       <c r="D97" t="inlineStr"/>
       <c r="E97" t="inlineStr"/>
-      <c r="F97" t="inlineStr">
-        <is>
-          <t>selected(${q1_21}, 'aterro_lixao')</t>
-        </is>
-      </c>
+      <c r="F97" t="inlineStr"/>
       <c r="G97" t="inlineStr"/>
       <c r="H97" t="inlineStr"/>
       <c r="I97" t="inlineStr"/>
@@ -3126,24 +3094,24 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>select_multiple relacao_elem</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>q1_22_10</t>
+          <t>q1_9r</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Áreas queimadas</t>
+          <t>Q1.9. Quem é responsável por esse monitoramento?</t>
         </is>
       </c>
       <c r="D98" t="inlineStr"/>
       <c r="E98" t="inlineStr"/>
       <c r="F98" t="inlineStr">
         <is>
-          <t>selected(${q1_21}, 'areas_queimadas')</t>
+          <t>${q1_8r} != '' and ${q1_8r} != 'em_nenhuma' and ${q1_8r} != 'nao_sabe'</t>
         </is>
       </c>
       <c r="G98" t="inlineStr"/>
@@ -3154,24 +3122,24 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>select_multiple relacao_elem</t>
+          <t>select_one sim_nao_ns</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>q1_22_11</t>
+          <t>q1_10r</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Áreas inundáveis</t>
+          <t>Q1.10. A secretaria/órgão tem acesso aos registros desse monitoramento?</t>
         </is>
       </c>
       <c r="D99" t="inlineStr"/>
       <c r="E99" t="inlineStr"/>
       <c r="F99" t="inlineStr">
         <is>
-          <t>selected(${q1_21}, 'areas_inundaveis')</t>
+          <t>${q1_8r} != '' and ${q1_8r} != 'em_nenhuma' and ${q1_8r} != 'nao_sabe'</t>
         </is>
       </c>
       <c r="G99" t="inlineStr"/>
@@ -3182,26 +3150,22 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>select_multiple relacao_elem</t>
+          <t>select_multiple infra_hidrica</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>q1_22_12</t>
+          <t>q1_11r</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Áreas degradadas</t>
+          <t>Q1.11. Infraestrutura hídrica presente nas escolas da rede</t>
         </is>
       </c>
       <c r="D100" t="inlineStr"/>
       <c r="E100" t="inlineStr"/>
-      <c r="F100" t="inlineStr">
-        <is>
-          <t>selected(${q1_21}, 'areas_degradadas')</t>
-        </is>
-      </c>
+      <c r="F100" t="inlineStr"/>
       <c r="G100" t="inlineStr"/>
       <c r="H100" t="inlineStr"/>
       <c r="I100" t="inlineStr"/>
@@ -3210,24 +3174,24 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>select_multiple relacao_elem</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>q1_22_13</t>
+          <t>q1_11r_outro</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Outros</t>
+          <t>Especifique (Outro)</t>
         </is>
       </c>
       <c r="D101" t="inlineStr"/>
       <c r="E101" t="inlineStr"/>
       <c r="F101" t="inlineStr">
         <is>
-          <t>selected(${q1_21}, 'outro')</t>
+          <t>selected(${q1_11r}, 'outro')</t>
         </is>
       </c>
       <c r="G101" t="inlineStr"/>
@@ -3238,11 +3202,19 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>end_group</t>
-        </is>
-      </c>
-      <c r="B102" t="inlineStr"/>
-      <c r="C102" t="inlineStr"/>
+          <t>select_multiple esgoto</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>q1_12r</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>Q1.12. Destinação do esgoto nas escolas da rede</t>
+        </is>
+      </c>
       <c r="D102" t="inlineStr"/>
       <c r="E102" t="inlineStr"/>
       <c r="F102" t="inlineStr"/>
@@ -3254,24 +3226,24 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>q1_22_nota</t>
+          <t>q1_12r_outro</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Nota para tutoria: um mesmo elemento pode ter mais de uma relação ao mesmo tempo (ex.: um rio pode ser, simultaneamente, ambiente e cultura, ou risco e uso comunitário) — marque quantas se aplicarem.</t>
+          <t>Especifique (Outro)</t>
         </is>
       </c>
       <c r="D103" t="inlineStr"/>
       <c r="E103" t="inlineStr"/>
       <c r="F103" t="inlineStr">
         <is>
-          <t>${q1_21} != ''</t>
+          <t>selected(${q1_12r}, 'outro')</t>
         </is>
       </c>
       <c r="G103" t="inlineStr"/>
@@ -3282,17 +3254,17 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>select_multiple ativ_econ</t>
+          <t>select_one qtd_rede</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>q1_23</t>
+          <t>q1_13r</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Q1.23. Principais atividades econômicas do território</t>
+          <t>Q1.13. Em quantas escolas da rede há esgoto a céu aberto no entorno?</t>
         </is>
       </c>
       <c r="D104" t="inlineStr"/>
@@ -3306,26 +3278,26 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>select_one qtd_rede</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>q1_23_outro</t>
+          <t>q1_14r</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Especifique (Outro)</t>
+          <t>Q1.14. Em quantas escolas da rede ocorrem alagamentos na escola ou no entorno?</t>
         </is>
       </c>
       <c r="D105" t="inlineStr"/>
-      <c r="E105" t="inlineStr"/>
-      <c r="F105" t="inlineStr">
-        <is>
-          <t>selected(${q1_23}, 'outro')</t>
-        </is>
-      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr"/>
       <c r="G105" t="inlineStr"/>
       <c r="H105" t="inlineStr"/>
       <c r="I105" t="inlineStr"/>
@@ -3334,23 +3306,31 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>select_one sim_nao_ns</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>q1_24</t>
+          <t>q1_15r</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Q1.24. Essas atividades têm impacto percebido no ambiente ou na comunidade?</t>
+          <t>Q1.15. Quais escolas/regiões são mais afetadas?</t>
         </is>
       </c>
       <c r="D106" t="inlineStr"/>
       <c r="E106" t="inlineStr"/>
-      <c r="F106" t="inlineStr"/>
-      <c r="G106" t="inlineStr"/>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>${q1_14r} != '' and ${q1_14r} != 'em_nenhuma' and ${q1_14r} != 'nao_sabe'</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>multiline</t>
+        </is>
+      </c>
       <c r="H106" t="inlineStr"/>
       <c r="I106" t="inlineStr"/>
       <c r="J106" t="inlineStr"/>
@@ -3358,31 +3338,27 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>select_multiple impacto_alag</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>q1_25</t>
+          <t>q1_16r</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Q1.25. Descreva os impactos percebidos por atividade</t>
+          <t>Q1.16. Impactos observados nesses episódios</t>
         </is>
       </c>
       <c r="D107" t="inlineStr"/>
       <c r="E107" t="inlineStr"/>
       <c r="F107" t="inlineStr">
         <is>
-          <t>${q1_24}='sim'</t>
-        </is>
-      </c>
-      <c r="G107" t="inlineStr">
-        <is>
-          <t>multiline</t>
-        </is>
-      </c>
+          <t>${q1_14r} != '' and ${q1_14r} != 'em_nenhuma' and ${q1_14r} != 'nao_sabe'</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr"/>
       <c r="H107" t="inlineStr"/>
       <c r="I107" t="inlineStr"/>
       <c r="J107" t="inlineStr"/>
@@ -3390,22 +3366,26 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>select_one sim_nao_ns</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>q1_26</t>
+          <t>q1_16r_outro</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Q1.26. Há eventos sazonais que afetam o local/comunidade (safras, secas, chuvas, festas, etc.)?</t>
+          <t>Especifique (Outro)</t>
         </is>
       </c>
       <c r="D108" t="inlineStr"/>
       <c r="E108" t="inlineStr"/>
-      <c r="F108" t="inlineStr"/>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>(${q1_14r} != '' and ${q1_14r} != 'em_nenhuma' and ${q1_14r} != 'nao_sabe') and selected(${q1_16r}, 'outro')</t>
+        </is>
+      </c>
       <c r="G108" t="inlineStr"/>
       <c r="H108" t="inlineStr"/>
       <c r="I108" t="inlineStr"/>
@@ -3414,31 +3394,23 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>select_one qtd_rede</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>q1_27</t>
+          <t>q1_17r</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Q1.27. Qual é esse evento? Descreva-o.</t>
+          <t>Q1.17. Em quantas escolas da rede há separação de resíduos?</t>
         </is>
       </c>
       <c r="D109" t="inlineStr"/>
       <c r="E109" t="inlineStr"/>
-      <c r="F109" t="inlineStr">
-        <is>
-          <t>${q1_26}='sim'</t>
-        </is>
-      </c>
-      <c r="G109" t="inlineStr">
-        <is>
-          <t>multiline</t>
-        </is>
-      </c>
+      <c r="F109" t="inlineStr"/>
+      <c r="G109" t="inlineStr"/>
       <c r="H109" t="inlineStr"/>
       <c r="I109" t="inlineStr"/>
       <c r="J109" t="inlineStr"/>
@@ -3446,26 +3418,22 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>select_multiple meses</t>
+          <t>select_multiple destino_res</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>q1_28</t>
+          <t>q1_18r</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>Q1.28. Em quais meses ele costuma ocorrer?</t>
+          <t>Q1.18. Destinação dos resíduos nas escolas da rede</t>
         </is>
       </c>
       <c r="D110" t="inlineStr"/>
       <c r="E110" t="inlineStr"/>
-      <c r="F110" t="inlineStr">
-        <is>
-          <t>${q1_26}='sim'</t>
-        </is>
-      </c>
+      <c r="F110" t="inlineStr"/>
       <c r="G110" t="inlineStr"/>
       <c r="H110" t="inlineStr"/>
       <c r="I110" t="inlineStr"/>
@@ -3479,26 +3447,22 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>q1_29</t>
+          <t>q1_18r_outro</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Q1.29. Qual o impacto desse evento neste local?</t>
+          <t>Especifique (Outro)</t>
         </is>
       </c>
       <c r="D111" t="inlineStr"/>
       <c r="E111" t="inlineStr"/>
       <c r="F111" t="inlineStr">
         <is>
-          <t>${q1_26}='sim'</t>
-        </is>
-      </c>
-      <c r="G111" t="inlineStr">
-        <is>
-          <t>multiline</t>
-        </is>
-      </c>
+          <t>selected(${q1_18r}, 'outro')</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr"/>
       <c r="H111" t="inlineStr"/>
       <c r="I111" t="inlineStr"/>
       <c r="J111" t="inlineStr"/>
@@ -3506,29 +3470,37 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>select_one sim_nao_ns</t>
+          <t>select_multiple prob_res</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>q1_30</t>
+          <t>q1_19r</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>Q1.30. Há histórico de eventos climáticos extremos que afetaram o local/comunidade?</t>
-        </is>
-      </c>
-      <c r="D112" t="inlineStr"/>
-      <c r="E112" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
+          <t>Q1.19. Problemas relacionados a resíduos no entorno das escolas da rede</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>Considere a área imediatamente ao redor das escolas, não o município inteiro.</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr"/>
       <c r="F112" t="inlineStr"/>
       <c r="G112" t="inlineStr"/>
-      <c r="H112" t="inlineStr"/>
-      <c r="I112" t="inlineStr"/>
+      <c r="H112" t="inlineStr">
+        <is>
+          <t>not((selected(., 'nenhum') or selected(., 'nao_sabe')) and count-selected(.) &gt; 1)</t>
+        </is>
+      </c>
+      <c r="I112" t="inlineStr">
+        <is>
+          <t>"Nenhum" e "Não sabe" não podem ser combinados com outras opções.</t>
+        </is>
+      </c>
       <c r="J112" t="inlineStr"/>
     </row>
     <row r="113">
@@ -3539,26 +3511,22 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>q1_31</t>
+          <t>q1_19r_outro</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Q1.31. Descreva o(s) evento(s)</t>
+          <t>Especifique (Outro)</t>
         </is>
       </c>
       <c r="D113" t="inlineStr"/>
       <c r="E113" t="inlineStr"/>
       <c r="F113" t="inlineStr">
         <is>
-          <t>${q1_30}='sim'</t>
-        </is>
-      </c>
-      <c r="G113" t="inlineStr">
-        <is>
-          <t>multiline</t>
-        </is>
-      </c>
+          <t>selected(${q1_19r}, 'outro')</t>
+        </is>
+      </c>
+      <c r="G113" t="inlineStr"/>
       <c r="H113" t="inlineStr"/>
       <c r="I113" t="inlineStr"/>
       <c r="J113" t="inlineStr"/>
@@ -3571,22 +3539,26 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>q1_32</t>
+          <t>q1_20r</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>Q1.32. Quando ocorreu(ram)?</t>
+          <t>Q1.20. Descreva esses problemas</t>
         </is>
       </c>
       <c r="D114" t="inlineStr"/>
       <c r="E114" t="inlineStr"/>
       <c r="F114" t="inlineStr">
         <is>
-          <t>${q1_30}='sim'</t>
-        </is>
-      </c>
-      <c r="G114" t="inlineStr"/>
+          <t>${q1_19r} != '' and not(selected(${q1_19r}, 'nenhum')) and not(selected(${q1_19r}, 'nao_sabe'))</t>
+        </is>
+      </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>multiline</t>
+        </is>
+      </c>
       <c r="H114" t="inlineStr"/>
       <c r="I114" t="inlineStr"/>
       <c r="J114" t="inlineStr"/>
@@ -3594,26 +3566,14 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>select_multiple impacto_clima</t>
-        </is>
-      </c>
-      <c r="B115" t="inlineStr">
-        <is>
-          <t>q1_33</t>
-        </is>
-      </c>
-      <c r="C115" t="inlineStr">
-        <is>
-          <t>Q1.33. Impactos observados</t>
-        </is>
-      </c>
+          <t>end_group</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr"/>
+      <c r="C115" t="inlineStr"/>
       <c r="D115" t="inlineStr"/>
       <c r="E115" t="inlineStr"/>
-      <c r="F115" t="inlineStr">
-        <is>
-          <t>${q1_30}='sim'</t>
-        </is>
-      </c>
+      <c r="F115" t="inlineStr"/>
       <c r="G115" t="inlineStr"/>
       <c r="H115" t="inlineStr"/>
       <c r="I115" t="inlineStr"/>
@@ -3622,26 +3582,30 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>select_multiple elementos</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>q1_33_outro</t>
+          <t>q1_21</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>Especifique (Outro)</t>
-        </is>
-      </c>
-      <c r="D116" t="inlineStr"/>
-      <c r="E116" t="inlineStr"/>
-      <c r="F116" t="inlineStr">
-        <is>
-          <t>(${q1_30}='sim') and selected(${q1_33}, 'outro')</t>
-        </is>
-      </c>
+          <t>Q1.21. Elementos presentes no território de atuação</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>Considere o território mais imediato — para uma local, o bairro ou a região do entorno em que a comunidade escolar circula; para uma secretaria ou regional, a área de abrangência da rede (não o município inteiro, se a atuação for menor). A existência de um elemento não significa, por si só, risco ou impacto — isso será explorado a seguir.</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr"/>
       <c r="G116" t="inlineStr"/>
       <c r="H116" t="inlineStr"/>
       <c r="I116" t="inlineStr"/>
@@ -3655,26 +3619,22 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>q1_34</t>
+          <t>q1_21_outro</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>Q1.34. O que o local/comunidade aprendeu com esse evento?</t>
+          <t>Especifique (Outro)</t>
         </is>
       </c>
       <c r="D117" t="inlineStr"/>
       <c r="E117" t="inlineStr"/>
       <c r="F117" t="inlineStr">
         <is>
-          <t>${q1_30}='sim'</t>
-        </is>
-      </c>
-      <c r="G117" t="inlineStr">
-        <is>
-          <t>multiline</t>
-        </is>
-      </c>
+          <t>selected(${q1_21}, 'outro')</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr"/>
       <c r="H117" t="inlineStr"/>
       <c r="I117" t="inlineStr"/>
       <c r="J117" t="inlineStr"/>
@@ -3682,29 +3642,29 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>begin_group</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>q1_35</t>
+          <t>t1_22</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>Q1.35. Quais são as características-chave deste território, na sua leitura?</t>
-        </is>
-      </c>
-      <c r="D118" t="inlineStr">
-        <is>
-          <t>Pense, por exemplo, em: relação com a água (rios, córregos, abastecimento), vegetação e áreas verdes, uso do solo predominante, memória e cultura local, riscos já percebidos e atividades econômicas mais presentes.</t>
-        </is>
-      </c>
+          <t>Q1.22. Para cada elemento selecionado, qual sua relação com o local/comunidade?</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr"/>
       <c r="E118" t="inlineStr"/>
-      <c r="F118" t="inlineStr"/>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>${q1_21} != ''</t>
+        </is>
+      </c>
       <c r="G118" t="inlineStr">
         <is>
-          <t>multiline</t>
+          <t>table-list</t>
         </is>
       </c>
       <c r="H118" t="inlineStr"/>
@@ -3714,31 +3674,27 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>select_multiple relacao_elem</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>q1_36</t>
+          <t>q1_22_01</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>Q1.36. Há algum aspecto do território que vocês reconhecem não saber ainda?</t>
-        </is>
-      </c>
-      <c r="D119" t="inlineStr">
-        <is>
-          <t>'Não sabemos' é uma resposta válida — isso vira uma lacuna de conhecimento registrada.</t>
-        </is>
-      </c>
+          <t>Rios/córregos</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr"/>
       <c r="E119" t="inlineStr"/>
-      <c r="F119" t="inlineStr"/>
-      <c r="G119" t="inlineStr">
-        <is>
-          <t>multiline</t>
-        </is>
-      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>selected(${q1_21}, 'rios_corregos')</t>
+        </is>
+      </c>
+      <c r="G119" t="inlineStr"/>
       <c r="H119" t="inlineStr"/>
       <c r="I119" t="inlineStr"/>
       <c r="J119" t="inlineStr"/>
@@ -3746,22 +3702,26 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>begin_repeat</t>
+          <t>select_multiple relacao_elem</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>evid_e1</t>
+          <t>q1_22_02</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>Evidências — Evidências sobre o local e o território</t>
+          <t>Lagoas/lagos/reservatórios</t>
         </is>
       </c>
       <c r="D120" t="inlineStr"/>
       <c r="E120" t="inlineStr"/>
-      <c r="F120" t="inlineStr"/>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>selected(${q1_21}, 'lagoas_lagos_reservatorios')</t>
+        </is>
+      </c>
       <c r="G120" t="inlineStr"/>
       <c r="H120" t="inlineStr"/>
       <c r="I120" t="inlineStr"/>
@@ -3770,22 +3730,26 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>select_multiple relacao_elem</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>evid_e1_nota</t>
+          <t>q1_22_03</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>Evidências sustentam análises futuras (problemas, prioridades, plano de ação). Registrar não é obrigatório para todo campo, mas fortalece a rastreabilidade do diagnóstico.</t>
+          <t>Vegetação</t>
         </is>
       </c>
       <c r="D121" t="inlineStr"/>
       <c r="E121" t="inlineStr"/>
-      <c r="F121" t="inlineStr"/>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>selected(${q1_21}, 'vegetacao')</t>
+        </is>
+      </c>
       <c r="G121" t="inlineStr"/>
       <c r="H121" t="inlineStr"/>
       <c r="I121" t="inlineStr"/>
@@ -3794,22 +3758,26 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>select_one tipo_evid</t>
+          <t>select_multiple relacao_elem</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>evid_e1_tipo</t>
+          <t>q1_22_04</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>Tipo de evidência</t>
+          <t>Parques</t>
         </is>
       </c>
       <c r="D122" t="inlineStr"/>
       <c r="E122" t="inlineStr"/>
-      <c r="F122" t="inlineStr"/>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>selected(${q1_21}, 'parques')</t>
+        </is>
+      </c>
       <c r="G122" t="inlineStr"/>
       <c r="H122" t="inlineStr"/>
       <c r="I122" t="inlineStr"/>
@@ -3818,24 +3786,24 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>select_multiple relacao_elem</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>evid_e1_tipo_outro</t>
+          <t>q1_22_05</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>Especifique (Outro)</t>
+          <t>Encostas</t>
         </is>
       </c>
       <c r="D123" t="inlineStr"/>
       <c r="E123" t="inlineStr"/>
       <c r="F123" t="inlineStr">
         <is>
-          <t>${evid_e1_tipo}='outro'</t>
+          <t>selected(${q1_21}, 'encostas')</t>
         </is>
       </c>
       <c r="G123" t="inlineStr"/>
@@ -3846,27 +3814,27 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>select_multiple relacao_elem</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>evid_e1_desc</t>
+          <t>q1_22_06</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>Descreva a evidência</t>
+          <t>Agricultura</t>
         </is>
       </c>
       <c r="D124" t="inlineStr"/>
       <c r="E124" t="inlineStr"/>
-      <c r="F124" t="inlineStr"/>
-      <c r="G124" t="inlineStr">
-        <is>
-          <t>multiline</t>
-        </is>
-      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>selected(${q1_21}, 'agricultura')</t>
+        </is>
+      </c>
+      <c r="G124" t="inlineStr"/>
       <c r="H124" t="inlineStr"/>
       <c r="I124" t="inlineStr"/>
       <c r="J124" t="inlineStr"/>
@@ -3874,22 +3842,26 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>file</t>
+          <t>select_multiple relacao_elem</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>evid_e1_anexo</t>
+          <t>q1_22_07</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>Anexo (foto/documento) — opcional</t>
+          <t>Indústria</t>
         </is>
       </c>
       <c r="D125" t="inlineStr"/>
       <c r="E125" t="inlineStr"/>
-      <c r="F125" t="inlineStr"/>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>selected(${q1_21}, 'industria')</t>
+        </is>
+      </c>
       <c r="G125" t="inlineStr"/>
       <c r="H125" t="inlineStr"/>
       <c r="I125" t="inlineStr"/>
@@ -3898,14 +3870,26 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>end_repeat</t>
-        </is>
-      </c>
-      <c r="B126" t="inlineStr"/>
-      <c r="C126" t="inlineStr"/>
+          <t>select_multiple relacao_elem</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>q1_22_08</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>Mineração</t>
+        </is>
+      </c>
       <c r="D126" t="inlineStr"/>
       <c r="E126" t="inlineStr"/>
-      <c r="F126" t="inlineStr"/>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>selected(${q1_21}, 'mineracao')</t>
+        </is>
+      </c>
       <c r="G126" t="inlineStr"/>
       <c r="H126" t="inlineStr"/>
       <c r="I126" t="inlineStr"/>
@@ -3914,18 +3898,834 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>end_group</t>
-        </is>
-      </c>
-      <c r="B127" t="inlineStr"/>
-      <c r="C127" t="inlineStr"/>
+          <t>select_multiple relacao_elem</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>q1_22_09</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>Aterro/lixão</t>
+        </is>
+      </c>
       <c r="D127" t="inlineStr"/>
       <c r="E127" t="inlineStr"/>
-      <c r="F127" t="inlineStr"/>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>selected(${q1_21}, 'aterro_lixao')</t>
+        </is>
+      </c>
       <c r="G127" t="inlineStr"/>
       <c r="H127" t="inlineStr"/>
       <c r="I127" t="inlineStr"/>
       <c r="J127" t="inlineStr"/>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>select_multiple relacao_elem</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>q1_22_10</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>Áreas queimadas</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr"/>
+      <c r="E128" t="inlineStr"/>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>selected(${q1_21}, 'areas_queimadas')</t>
+        </is>
+      </c>
+      <c r="G128" t="inlineStr"/>
+      <c r="H128" t="inlineStr"/>
+      <c r="I128" t="inlineStr"/>
+      <c r="J128" t="inlineStr"/>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>select_multiple relacao_elem</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>q1_22_11</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>Áreas inundáveis</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr"/>
+      <c r="E129" t="inlineStr"/>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>selected(${q1_21}, 'areas_inundaveis')</t>
+        </is>
+      </c>
+      <c r="G129" t="inlineStr"/>
+      <c r="H129" t="inlineStr"/>
+      <c r="I129" t="inlineStr"/>
+      <c r="J129" t="inlineStr"/>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>select_multiple relacao_elem</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>q1_22_12</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>Áreas degradadas</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr"/>
+      <c r="E130" t="inlineStr"/>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>selected(${q1_21}, 'areas_degradadas')</t>
+        </is>
+      </c>
+      <c r="G130" t="inlineStr"/>
+      <c r="H130" t="inlineStr"/>
+      <c r="I130" t="inlineStr"/>
+      <c r="J130" t="inlineStr"/>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>select_multiple relacao_elem</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>q1_22_13</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>Outros</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr"/>
+      <c r="E131" t="inlineStr"/>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>selected(${q1_21}, 'outro')</t>
+        </is>
+      </c>
+      <c r="G131" t="inlineStr"/>
+      <c r="H131" t="inlineStr"/>
+      <c r="I131" t="inlineStr"/>
+      <c r="J131" t="inlineStr"/>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>end_group</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr"/>
+      <c r="C132" t="inlineStr"/>
+      <c r="D132" t="inlineStr"/>
+      <c r="E132" t="inlineStr"/>
+      <c r="F132" t="inlineStr"/>
+      <c r="G132" t="inlineStr"/>
+      <c r="H132" t="inlineStr"/>
+      <c r="I132" t="inlineStr"/>
+      <c r="J132" t="inlineStr"/>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>q1_22_nota</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>Nota para tutoria: um mesmo elemento pode ter mais de uma relação ao mesmo tempo (ex.: um rio pode ser, simultaneamente, ambiente e cultura, ou risco e uso comunitário) — marque quantas se aplicarem.</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr"/>
+      <c r="E133" t="inlineStr"/>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>${q1_21} != ''</t>
+        </is>
+      </c>
+      <c r="G133" t="inlineStr"/>
+      <c r="H133" t="inlineStr"/>
+      <c r="I133" t="inlineStr"/>
+      <c r="J133" t="inlineStr"/>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>select_multiple ativ_econ</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>q1_23</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>Q1.23. Principais atividades econômicas do território</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr"/>
+      <c r="E134" t="inlineStr"/>
+      <c r="F134" t="inlineStr"/>
+      <c r="G134" t="inlineStr"/>
+      <c r="H134" t="inlineStr"/>
+      <c r="I134" t="inlineStr"/>
+      <c r="J134" t="inlineStr"/>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>q1_23_outro</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>Especifique (Outro)</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr"/>
+      <c r="E135" t="inlineStr"/>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>selected(${q1_23}, 'outro')</t>
+        </is>
+      </c>
+      <c r="G135" t="inlineStr"/>
+      <c r="H135" t="inlineStr"/>
+      <c r="I135" t="inlineStr"/>
+      <c r="J135" t="inlineStr"/>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>select_one sim_nao_ns</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>q1_24</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>Q1.24. Essas atividades têm impacto percebido no ambiente ou na comunidade?</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr"/>
+      <c r="E136" t="inlineStr"/>
+      <c r="F136" t="inlineStr"/>
+      <c r="G136" t="inlineStr"/>
+      <c r="H136" t="inlineStr"/>
+      <c r="I136" t="inlineStr"/>
+      <c r="J136" t="inlineStr"/>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>q1_25</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>Q1.25. Descreva os impactos percebidos por atividade</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr"/>
+      <c r="E137" t="inlineStr"/>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>${q1_24}='sim'</t>
+        </is>
+      </c>
+      <c r="G137" t="inlineStr">
+        <is>
+          <t>multiline</t>
+        </is>
+      </c>
+      <c r="H137" t="inlineStr"/>
+      <c r="I137" t="inlineStr"/>
+      <c r="J137" t="inlineStr"/>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>select_one sim_nao_ns</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>q1_26</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>Q1.26. Há eventos sazonais que afetam o local/comunidade (safras, secas, chuvas, festas, etc.)?</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr"/>
+      <c r="E138" t="inlineStr"/>
+      <c r="F138" t="inlineStr"/>
+      <c r="G138" t="inlineStr"/>
+      <c r="H138" t="inlineStr"/>
+      <c r="I138" t="inlineStr"/>
+      <c r="J138" t="inlineStr"/>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>q1_27</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>Q1.27. Qual é esse evento? Descreva-o.</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr"/>
+      <c r="E139" t="inlineStr"/>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>${q1_26}='sim'</t>
+        </is>
+      </c>
+      <c r="G139" t="inlineStr">
+        <is>
+          <t>multiline</t>
+        </is>
+      </c>
+      <c r="H139" t="inlineStr"/>
+      <c r="I139" t="inlineStr"/>
+      <c r="J139" t="inlineStr"/>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>select_multiple meses</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>q1_28</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>Q1.28. Em quais meses ele costuma ocorrer?</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr"/>
+      <c r="E140" t="inlineStr"/>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t>${q1_26}='sim'</t>
+        </is>
+      </c>
+      <c r="G140" t="inlineStr"/>
+      <c r="H140" t="inlineStr"/>
+      <c r="I140" t="inlineStr"/>
+      <c r="J140" t="inlineStr"/>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>q1_29</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>Q1.29. Qual o impacto desse evento neste local?</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr"/>
+      <c r="E141" t="inlineStr"/>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>${q1_26}='sim'</t>
+        </is>
+      </c>
+      <c r="G141" t="inlineStr">
+        <is>
+          <t>multiline</t>
+        </is>
+      </c>
+      <c r="H141" t="inlineStr"/>
+      <c r="I141" t="inlineStr"/>
+      <c r="J141" t="inlineStr"/>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>select_one sim_nao_ns</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>q1_30</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>Q1.30. Há histórico de eventos climáticos extremos que afetaram o local/comunidade?</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr"/>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="F142" t="inlineStr"/>
+      <c r="G142" t="inlineStr"/>
+      <c r="H142" t="inlineStr"/>
+      <c r="I142" t="inlineStr"/>
+      <c r="J142" t="inlineStr"/>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>q1_31</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>Q1.31. Descreva o(s) evento(s)</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr"/>
+      <c r="E143" t="inlineStr"/>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t>${q1_30}='sim'</t>
+        </is>
+      </c>
+      <c r="G143" t="inlineStr">
+        <is>
+          <t>multiline</t>
+        </is>
+      </c>
+      <c r="H143" t="inlineStr"/>
+      <c r="I143" t="inlineStr"/>
+      <c r="J143" t="inlineStr"/>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>q1_32</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>Q1.32. Quando ocorreu(ram)?</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr"/>
+      <c r="E144" t="inlineStr"/>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>${q1_30}='sim'</t>
+        </is>
+      </c>
+      <c r="G144" t="inlineStr"/>
+      <c r="H144" t="inlineStr"/>
+      <c r="I144" t="inlineStr"/>
+      <c r="J144" t="inlineStr"/>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>select_multiple impacto_clima</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>q1_33</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>Q1.33. Impactos observados</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr"/>
+      <c r="E145" t="inlineStr"/>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>${q1_30}='sim'</t>
+        </is>
+      </c>
+      <c r="G145" t="inlineStr"/>
+      <c r="H145" t="inlineStr"/>
+      <c r="I145" t="inlineStr"/>
+      <c r="J145" t="inlineStr"/>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>q1_33_outro</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>Especifique (Outro)</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr"/>
+      <c r="E146" t="inlineStr"/>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>(${q1_30}='sim') and selected(${q1_33}, 'outro')</t>
+        </is>
+      </c>
+      <c r="G146" t="inlineStr"/>
+      <c r="H146" t="inlineStr"/>
+      <c r="I146" t="inlineStr"/>
+      <c r="J146" t="inlineStr"/>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>q1_34</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>Q1.34. O que o local/comunidade aprendeu com esse evento?</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr"/>
+      <c r="E147" t="inlineStr"/>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>${q1_30}='sim'</t>
+        </is>
+      </c>
+      <c r="G147" t="inlineStr">
+        <is>
+          <t>multiline</t>
+        </is>
+      </c>
+      <c r="H147" t="inlineStr"/>
+      <c r="I147" t="inlineStr"/>
+      <c r="J147" t="inlineStr"/>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>q1_35</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>Q1.35. Quais são as características-chave deste território, na sua leitura?</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>Pense, por exemplo, em: relação com a água (rios, córregos, abastecimento), vegetação e áreas verdes, uso do solo predominante, memória e cultura local, riscos já percebidos e atividades econômicas mais presentes.</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr"/>
+      <c r="F148" t="inlineStr"/>
+      <c r="G148" t="inlineStr">
+        <is>
+          <t>multiline</t>
+        </is>
+      </c>
+      <c r="H148" t="inlineStr"/>
+      <c r="I148" t="inlineStr"/>
+      <c r="J148" t="inlineStr"/>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>q1_36</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>Q1.36. Há algum aspecto do território que vocês reconhecem não saber ainda?</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>'Não sabemos' é uma resposta válida — isso vira uma lacuna de conhecimento registrada.</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr"/>
+      <c r="F149" t="inlineStr"/>
+      <c r="G149" t="inlineStr">
+        <is>
+          <t>multiline</t>
+        </is>
+      </c>
+      <c r="H149" t="inlineStr"/>
+      <c r="I149" t="inlineStr"/>
+      <c r="J149" t="inlineStr"/>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>begin_repeat</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>evid_e1</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>Evidências — Evidências sobre o local e o território</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr"/>
+      <c r="E150" t="inlineStr"/>
+      <c r="F150" t="inlineStr"/>
+      <c r="G150" t="inlineStr"/>
+      <c r="H150" t="inlineStr"/>
+      <c r="I150" t="inlineStr"/>
+      <c r="J150" t="inlineStr"/>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>evid_e1_nota</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>Evidências sustentam análises futuras (problemas, prioridades, plano de ação). Registrar não é obrigatório para todo campo, mas fortalece a rastreabilidade do diagnóstico.</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr"/>
+      <c r="E151" t="inlineStr"/>
+      <c r="F151" t="inlineStr"/>
+      <c r="G151" t="inlineStr"/>
+      <c r="H151" t="inlineStr"/>
+      <c r="I151" t="inlineStr"/>
+      <c r="J151" t="inlineStr"/>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>select_one tipo_evid</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>evid_e1_tipo</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>Tipo de evidência</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr"/>
+      <c r="E152" t="inlineStr"/>
+      <c r="F152" t="inlineStr"/>
+      <c r="G152" t="inlineStr"/>
+      <c r="H152" t="inlineStr"/>
+      <c r="I152" t="inlineStr"/>
+      <c r="J152" t="inlineStr"/>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>evid_e1_tipo_outro</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>Especifique (Outro)</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr"/>
+      <c r="E153" t="inlineStr"/>
+      <c r="F153" t="inlineStr">
+        <is>
+          <t>${evid_e1_tipo}='outro'</t>
+        </is>
+      </c>
+      <c r="G153" t="inlineStr"/>
+      <c r="H153" t="inlineStr"/>
+      <c r="I153" t="inlineStr"/>
+      <c r="J153" t="inlineStr"/>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>evid_e1_desc</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>Descreva a evidência</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr"/>
+      <c r="E154" t="inlineStr"/>
+      <c r="F154" t="inlineStr"/>
+      <c r="G154" t="inlineStr">
+        <is>
+          <t>multiline</t>
+        </is>
+      </c>
+      <c r="H154" t="inlineStr"/>
+      <c r="I154" t="inlineStr"/>
+      <c r="J154" t="inlineStr"/>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>file</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>evid_e1_anexo</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>Anexo (foto/documento) — opcional</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr"/>
+      <c r="E155" t="inlineStr"/>
+      <c r="F155" t="inlineStr"/>
+      <c r="G155" t="inlineStr"/>
+      <c r="H155" t="inlineStr"/>
+      <c r="I155" t="inlineStr"/>
+      <c r="J155" t="inlineStr"/>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>end_repeat</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr"/>
+      <c r="C156" t="inlineStr"/>
+      <c r="D156" t="inlineStr"/>
+      <c r="E156" t="inlineStr"/>
+      <c r="F156" t="inlineStr"/>
+      <c r="G156" t="inlineStr"/>
+      <c r="H156" t="inlineStr"/>
+      <c r="I156" t="inlineStr"/>
+      <c r="J156" t="inlineStr"/>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>end_group</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr"/>
+      <c r="C157" t="inlineStr"/>
+      <c r="D157" t="inlineStr"/>
+      <c r="E157" t="inlineStr"/>
+      <c r="F157" t="inlineStr"/>
+      <c r="G157" t="inlineStr"/>
+      <c r="H157" t="inlineStr"/>
+      <c r="I157" t="inlineStr"/>
+      <c r="J157" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Q1.1: adiciona opção Não se aplica
</commit_message>
<xml_diff>
--- a/kobo/gestores_semana1_diagnostico.xlsx
+++ b/kobo/gestores_semana1_diagnostico.xlsx
@@ -1750,7 +1750,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>select_one qtd_rede</t>
+          <t>select_one qtd_rede_tab</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1778,7 +1778,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>select_one qtd_rede</t>
+          <t>select_one qtd_rede_tab</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -1806,7 +1806,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>select_one qtd_rede</t>
+          <t>select_one qtd_rede_tab</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -1834,7 +1834,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>select_one qtd_rede</t>
+          <t>select_one qtd_rede_tab</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -1862,7 +1862,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>select_one qtd_rede</t>
+          <t>select_one qtd_rede_tab</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -1890,7 +1890,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>select_one qtd_rede</t>
+          <t>select_one qtd_rede_tab</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -1918,7 +1918,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>select_one qtd_rede</t>
+          <t>select_one qtd_rede_tab</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -1946,7 +1946,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>select_one qtd_rede</t>
+          <t>select_one qtd_rede_tab</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -1974,7 +1974,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>select_one qtd_rede</t>
+          <t>select_one qtd_rede_tab</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -2002,7 +2002,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>select_one qtd_rede</t>
+          <t>select_one qtd_rede_tab</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -2030,7 +2030,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>select_one qtd_rede</t>
+          <t>select_one qtd_rede_tab</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -4734,7 +4734,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C177"/>
+  <dimension ref="A1:C185"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6037,29 +6037,29 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>nao_sabe</t>
+          <t>nao_se_aplica</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Não sabe</t>
+          <t>Não se aplica</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>qtd_rede</t>
+          <t>estado_infra</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>em_nenhuma</t>
+          <t>nao_sabe</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Em nenhuma</t>
+          <t>Não sabe</t>
         </is>
       </c>
     </row>
@@ -6071,12 +6071,12 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>em_poucas</t>
+          <t>em_nenhuma</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Em poucas</t>
+          <t>Em nenhuma</t>
         </is>
       </c>
     </row>
@@ -6088,12 +6088,12 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>em_cerca_de_metade</t>
+          <t>em_poucas</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Em cerca de metade</t>
+          <t>Em poucas</t>
         </is>
       </c>
     </row>
@@ -6105,12 +6105,12 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>na_maioria</t>
+          <t>em_cerca_de_metade</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Na maioria</t>
+          <t>Em cerca de metade</t>
         </is>
       </c>
     </row>
@@ -6122,12 +6122,12 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>em_todas</t>
+          <t>na_maioria</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Em todas</t>
+          <t>Na maioria</t>
         </is>
       </c>
     </row>
@@ -6139,716 +6139,716 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>nao_sabe</t>
+          <t>em_todas</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Não sabe</t>
+          <t>Em todas</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>termica</t>
+          <t>qtd_rede</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>muito_quente_no_verao</t>
+          <t>nao_sabe</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Muito quente no verão</t>
+          <t>Não sabe</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>termica</t>
+          <t>qtd_rede_tab</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>muito_fria_no_inverno</t>
+          <t>em_nenhuma</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Muito fria no inverno</t>
+          <t>Em nenhuma</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>termica</t>
+          <t>qtd_rede_tab</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>adequada_na_maior_parte_do_ano</t>
+          <t>em_poucas</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Adequada na maior parte do ano</t>
+          <t>Em poucas</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>termica</t>
+          <t>qtd_rede_tab</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>muito_variavel_sem_padrao_sazona</t>
+          <t>em_cerca_de_metade</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Muito variável, sem padrão sazonal claro</t>
+          <t>Em cerca de metade</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>termica</t>
+          <t>qtd_rede_tab</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>nao_sabe</t>
+          <t>na_maioria</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Não sabe</t>
+          <t>Na maioria</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>prob_estrut</t>
+          <t>qtd_rede_tab</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>mofo</t>
+          <t>em_todas</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Mofo</t>
+          <t>Em todas</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>prob_estrut</t>
+          <t>qtd_rede_tab</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>infiltracao</t>
+          <t>nao_se_aplica</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Infiltração</t>
+          <t>Não se aplica</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>prob_estrut</t>
+          <t>qtd_rede_tab</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>calor_excessivo</t>
+          <t>nao_sabe</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Calor excessivo</t>
+          <t>Não sabe</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>prob_estrut</t>
+          <t>termica</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>frio_excessivo</t>
+          <t>muito_quente_no_verao</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Frio excessivo</t>
+          <t>Muito quente no verão</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>prob_estrut</t>
+          <t>termica</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>falta_de_ventilacao</t>
+          <t>muito_fria_no_inverno</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Falta de ventilação</t>
+          <t>Muito fria no inverno</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>prob_estrut</t>
+          <t>termica</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>outro</t>
+          <t>adequada_na_maior_parte_do_ano</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Outro</t>
+          <t>Adequada na maior parte do ano</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>agua_fonte</t>
+          <t>termica</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>rede_publica</t>
+          <t>muito_variavel_sem_padrao_sazona</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Rede pública</t>
+          <t>Muito variável, sem padrão sazonal claro</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>agua_fonte</t>
+          <t>termica</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>poco</t>
+          <t>nao_sabe</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Poço</t>
+          <t>Não sabe</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>agua_fonte</t>
+          <t>prob_estrut</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>nascente</t>
+          <t>mofo</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Nascente</t>
+          <t>Mofo</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>agua_fonte</t>
+          <t>prob_estrut</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>cisterna</t>
+          <t>infiltracao</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Cisterna</t>
+          <t>Infiltração</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>agua_fonte</t>
+          <t>prob_estrut</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>outro</t>
+          <t>calor_excessivo</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Outra</t>
+          <t>Calor excessivo</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>agua_fonte</t>
+          <t>prob_estrut</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>nao_sabe</t>
+          <t>frio_excessivo</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Não sabe</t>
+          <t>Frio excessivo</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>infra_hidrica</t>
+          <t>prob_estrut</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>reservatorio_caixa_d_agua</t>
+          <t>falta_de_ventilacao</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Reservatório / caixa d'água</t>
+          <t>Falta de ventilação</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>infra_hidrica</t>
+          <t>prob_estrut</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>filtro_purificador</t>
+          <t>outro</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Filtro / purificador</t>
+          <t>Outro</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>infra_hidrica</t>
+          <t>agua_fonte</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>bebedouros</t>
+          <t>rede_publica</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Bebedouros</t>
+          <t>Rede pública</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>infra_hidrica</t>
+          <t>agua_fonte</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>rede_encanada_interna</t>
+          <t>poco</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Rede encanada interna</t>
+          <t>Poço</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>infra_hidrica</t>
+          <t>agua_fonte</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>outro</t>
+          <t>nascente</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Outro</t>
+          <t>Nascente</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>infra_hidrica</t>
+          <t>agua_fonte</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>nao_sabe</t>
+          <t>cisterna</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Não sabe</t>
+          <t>Cisterna</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>esgoto</t>
+          <t>agua_fonte</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>rede_coletora</t>
+          <t>outro</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Rede coletora</t>
+          <t>Outra</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>esgoto</t>
+          <t>agua_fonte</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>fossa_septica</t>
+          <t>nao_sabe</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Fossa séptica</t>
+          <t>Não sabe</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>esgoto</t>
+          <t>infra_hidrica</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>fossa_rudimentar</t>
+          <t>reservatorio_caixa_d_agua</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Fossa rudimentar</t>
+          <t>Reservatório / caixa d'água</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>esgoto</t>
+          <t>infra_hidrica</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>ceu_aberto</t>
+          <t>filtro_purificador</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>Céu aberto</t>
+          <t>Filtro / purificador</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>esgoto</t>
+          <t>infra_hidrica</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>outro</t>
+          <t>bebedouros</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Outro</t>
+          <t>Bebedouros</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>esgoto</t>
+          <t>infra_hidrica</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>nao_sabe</t>
+          <t>rede_encanada_interna</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>Não sabe</t>
+          <t>Rede encanada interna</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>impacto_alag</t>
+          <t>infra_hidrica</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>interrupcao_de_aulas</t>
+          <t>outro</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Interrupção de aulas</t>
+          <t>Outro</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>impacto_alag</t>
+          <t>infra_hidrica</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>danos_a_estrutura</t>
+          <t>nao_sabe</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>Danos à estrutura</t>
+          <t>Não sabe</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>impacto_alag</t>
+          <t>esgoto</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>acesso_interrompido</t>
+          <t>rede_coletora</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>Dificuldade ou interrupção do acesso ao local</t>
+          <t>Rede coletora</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>impacto_alag</t>
+          <t>esgoto</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>baixa_adesao</t>
+          <t>fossa_septica</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>Baixa adesão dos estudantes (aulas mantidas, mas poucos conseguem frequentar)</t>
+          <t>Fossa séptica</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>impacto_alag</t>
+          <t>esgoto</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>outro</t>
+          <t>fossa_rudimentar</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>Outro</t>
+          <t>Fossa rudimentar</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>destino_res</t>
+          <t>esgoto</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>coleta_publica</t>
+          <t>ceu_aberto</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>Coleta pública</t>
+          <t>Céu aberto</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>destino_res</t>
+          <t>esgoto</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>coleta_seletiva</t>
+          <t>outro</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>Coleta seletiva</t>
+          <t>Outro</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>destino_res</t>
+          <t>esgoto</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>cooperativa</t>
+          <t>nao_sabe</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>Cooperativa</t>
+          <t>Não sabe</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>destino_res</t>
+          <t>impacto_alag</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>compostagem</t>
+          <t>interrupcao_de_aulas</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>Compostagem</t>
+          <t>Interrupção de aulas</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>destino_res</t>
+          <t>impacto_alag</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>reutilizacao</t>
+          <t>danos_a_estrutura</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>Reutilização</t>
+          <t>Danos à estrutura</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>destino_res</t>
+          <t>impacto_alag</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>queima</t>
+          <t>acesso_interrompido</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>Queima</t>
+          <t>Dificuldade ou interrupção do acesso ao local</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>destino_res</t>
+          <t>impacto_alag</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>enterramento</t>
+          <t>baixa_adesao</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>Enterramento</t>
+          <t>Baixa adesão dos estudantes (aulas mantidas, mas poucos conseguem frequentar)</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>destino_res</t>
+          <t>impacto_alag</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -6870,267 +6870,267 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>nao_sabe</t>
+          <t>coleta_publica</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>Não sabe</t>
+          <t>Coleta pública</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>prob_res</t>
+          <t>destino_res</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>aterro_sanitario</t>
+          <t>coleta_seletiva</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>Aterro sanitário</t>
+          <t>Coleta seletiva</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>prob_res</t>
+          <t>destino_res</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>lixao</t>
+          <t>cooperativa</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>Lixão</t>
+          <t>Cooperativa</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>prob_res</t>
+          <t>destino_res</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>queima_de_residuos</t>
+          <t>compostagem</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>Queima de resíduos</t>
+          <t>Compostagem</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>prob_res</t>
+          <t>destino_res</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>acumulo_de_residuos_no_entorno</t>
+          <t>reutilizacao</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>Acúmulo de resíduos no entorno</t>
+          <t>Reutilização</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>prob_res</t>
+          <t>destino_res</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>outro</t>
+          <t>queima</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>Outro</t>
+          <t>Queima</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>prob_res</t>
+          <t>destino_res</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>nenhum</t>
+          <t>enterramento</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>Nenhum</t>
+          <t>Enterramento</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>prob_res</t>
+          <t>destino_res</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>nao_sabe</t>
+          <t>outro</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>Não sabe</t>
+          <t>Outro</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>elementos</t>
+          <t>destino_res</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>rios_corregos</t>
+          <t>nao_sabe</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>Rios/córregos</t>
+          <t>Não sabe</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>elementos</t>
+          <t>prob_res</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>lagoas_lagos_reservatorios</t>
+          <t>aterro_sanitario</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>Lagoas/lagos/reservatórios</t>
+          <t>Aterro sanitário</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>elementos</t>
+          <t>prob_res</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>areas_de_vegetacao_nativa</t>
+          <t>lixao</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>Áreas de vegetação nativa (matas, florestas, campos)</t>
+          <t>Lixão</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>elementos</t>
+          <t>prob_res</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>parques</t>
+          <t>queima_de_residuos</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>Parques</t>
+          <t>Queima de resíduos</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>elementos</t>
+          <t>prob_res</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>encostas</t>
+          <t>acumulo_de_residuos_no_entorno</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>Encostas</t>
+          <t>Acúmulo de resíduos no entorno</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>elementos</t>
+          <t>prob_res</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>agricultura</t>
+          <t>outro</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>Agricultura</t>
+          <t>Outro</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>elementos</t>
+          <t>prob_res</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>industria</t>
+          <t>nenhum</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>Indústria</t>
+          <t>Nenhum</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>elementos</t>
+          <t>prob_res</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>mineracao</t>
+          <t>nao_sabe</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>Mineração</t>
+          <t>Não sabe</t>
         </is>
       </c>
     </row>
@@ -7142,12 +7142,12 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>aterro_lixao</t>
+          <t>rios_corregos</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>Aterro/lixão</t>
+          <t>Rios/córregos</t>
         </is>
       </c>
     </row>
@@ -7159,12 +7159,12 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>areas_queimadas</t>
+          <t>lagoas_lagos_reservatorios</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>Áreas queimadas</t>
+          <t>Lagoas/lagos/reservatórios</t>
         </is>
       </c>
     </row>
@@ -7176,12 +7176,12 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>areas_inundaveis</t>
+          <t>areas_de_vegetacao_nativa</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>Áreas inundáveis</t>
+          <t>Áreas de vegetação nativa (matas, florestas, campos)</t>
         </is>
       </c>
     </row>
@@ -7193,12 +7193,12 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>comercios</t>
+          <t>parques</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>Comércios</t>
+          <t>Parques</t>
         </is>
       </c>
     </row>
@@ -7210,12 +7210,12 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>outras_areas_degradadas</t>
+          <t>encostas</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>Outras áreas degradadas</t>
+          <t>Encostas</t>
         </is>
       </c>
     </row>
@@ -7227,12 +7227,12 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>equipamentos_urbanos</t>
+          <t>agricultura</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>Equipamentos Urbanos</t>
+          <t>Agricultura</t>
         </is>
       </c>
     </row>
@@ -7244,138 +7244,138 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>outro</t>
+          <t>industria</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>Outros</t>
+          <t>Indústria</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>relacao_elem</t>
+          <t>elementos</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>ambiente</t>
+          <t>mineracao</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>Ambiente</t>
+          <t>Mineração</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>relacao_elem</t>
+          <t>elementos</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>cultura</t>
+          <t>aterro_lixao</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>Cultura</t>
+          <t>Aterro/lixão</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>relacao_elem</t>
+          <t>elementos</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>uso_comunitario</t>
+          <t>areas_queimadas</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>Uso comunitário</t>
+          <t>Áreas queimadas</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>relacao_elem</t>
+          <t>elementos</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>renda</t>
+          <t>areas_inundaveis</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>Renda</t>
+          <t>Áreas inundáveis</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>relacao_elem</t>
+          <t>elementos</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>risco</t>
+          <t>comercios</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>Risco</t>
+          <t>Comércios</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>relacao_elem</t>
+          <t>elementos</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>degradacao</t>
+          <t>outras_areas_degradadas</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>Degradação</t>
+          <t>Outras áreas degradadas</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>relacao_elem</t>
+          <t>elementos</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>conflito</t>
+          <t>equipamentos_urbanos</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>Conflito</t>
+          <t>Equipamentos Urbanos</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>relacao_elem</t>
+          <t>elementos</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
@@ -7385,7 +7385,7 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>Outra</t>
+          <t>Outros</t>
         </is>
       </c>
     </row>
@@ -7397,350 +7397,486 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>nao_sabe</t>
+          <t>ambiente</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>Não sabe</t>
+          <t>Ambiente</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>ativ_econ</t>
+          <t>relacao_elem</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>agricultura</t>
+          <t>cultura</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>Agricultura</t>
+          <t>Cultura</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>ativ_econ</t>
+          <t>relacao_elem</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>pecuaria</t>
+          <t>uso_comunitario</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>Pecuária</t>
+          <t>Uso comunitário</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>ativ_econ</t>
+          <t>relacao_elem</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>comercio</t>
+          <t>renda</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>Comércio</t>
+          <t>Renda</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>ativ_econ</t>
+          <t>relacao_elem</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>industria</t>
+          <t>risco</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>Indústria</t>
+          <t>Risco</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>ativ_econ</t>
+          <t>relacao_elem</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>turismo</t>
+          <t>degradacao</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>Turismo</t>
+          <t>Degradação</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>ativ_econ</t>
+          <t>relacao_elem</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>pesca</t>
+          <t>conflito</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>Pesca</t>
+          <t>Conflito</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>ativ_econ</t>
+          <t>relacao_elem</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>extrativismo</t>
+          <t>outro</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>Extrativismo</t>
+          <t>Outra</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>ativ_econ</t>
+          <t>relacao_elem</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>outro</t>
+          <t>nao_sabe</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>Outro</t>
+          <t>Não sabe</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>impacto_clima</t>
+          <t>ativ_econ</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>interrupcao_de_aulas</t>
+          <t>agricultura</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>Interrupção de aulas</t>
+          <t>Agricultura</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>impacto_clima</t>
+          <t>ativ_econ</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>danos_materiais</t>
+          <t>pecuaria</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>Danos materiais</t>
+          <t>Pecuária</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>impacto_clima</t>
+          <t>ativ_econ</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>deslocamento_de_pessoas</t>
+          <t>comercio</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>Deslocamento de pessoas (necessidade de migração)</t>
+          <t>Comércio</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>impacto_clima</t>
+          <t>ativ_econ</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>perdas</t>
+          <t>industria</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>Óbitos</t>
+          <t>Indústria</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>impacto_clima</t>
+          <t>ativ_econ</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>impacto_emocional</t>
+          <t>turismo</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>Impacto emocional</t>
+          <t>Turismo</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>impacto_clima</t>
+          <t>ativ_econ</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>outro</t>
+          <t>pesca</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>Outro</t>
+          <t>Pesca</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>tipo_evid</t>
+          <t>ativ_econ</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>observacao_direta</t>
+          <t>extrativismo</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>Observação direta</t>
+          <t>Extrativismo</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>tipo_evid</t>
+          <t>ativ_econ</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>documento</t>
+          <t>outro</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>Documento</t>
+          <t>Outro</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>tipo_evid</t>
+          <t>impacto_clima</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>foto</t>
+          <t>interrupcao_de_aulas</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>Foto</t>
+          <t>Interrupção de aulas</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>tipo_evid</t>
+          <t>impacto_clima</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>depoimento</t>
+          <t>danos_materiais</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>Depoimento</t>
+          <t>Danos materiais</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>tipo_evid</t>
+          <t>impacto_clima</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>registro_historico</t>
+          <t>deslocamento_de_pessoas</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>Registro histórico</t>
+          <t>Deslocamento de pessoas (necessidade de migração)</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
+          <t>impacto_clima</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>perdas</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>Óbitos</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>impacto_clima</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>impacto_emocional</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>Impacto emocional</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>impacto_clima</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>outro</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>Outro</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
           <t>tipo_evid</t>
         </is>
       </c>
-      <c r="B177" t="inlineStr">
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>observacao_direta</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>Observação direta</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>tipo_evid</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>documento</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>Documento</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>tipo_evid</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>foto</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>Foto</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>tipo_evid</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>depoimento</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>Depoimento</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>tipo_evid</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>registro_historico</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>Registro histórico</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>tipo_evid</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
         <is>
           <t>outro</t>
         </is>
       </c>
-      <c r="C177" t="inlineStr">
+      <c r="C185" t="inlineStr">
         <is>
           <t>Outra</t>
         </is>

</xml_diff>

<commit_message>
Etapa 1: controle térmico, exemplos de eventos extremos e impactos positivos
</commit_message>
<xml_diff>
--- a/kobo/gestores_semana1_diagnostico.xlsx
+++ b/kobo/gestores_semana1_diagnostico.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J158"/>
+  <dimension ref="A1:J162"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1702,13 +1702,25 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>end_group</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr"/>
-      <c r="C47" t="inlineStr"/>
+          <t>select_one estado_infra</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>q1_1_12</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Ar-condicionado nas salas de aula</t>
+        </is>
+      </c>
       <c r="D47" t="inlineStr"/>
-      <c r="E47" t="inlineStr"/>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
       <c r="F47" t="inlineStr"/>
       <c r="G47" t="inlineStr"/>
       <c r="H47" t="inlineStr"/>
@@ -1718,31 +1730,27 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>begin_group</t>
+          <t>select_one estado_infra</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>t1_1r</t>
+          <t>q1_1_13</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Q1.1. Infraestrutura da rede — em quantas escolas da rede existe cada espaço?</t>
+          <t>Ventiladores/estufas nas salas de aula</t>
         </is>
       </c>
       <c r="D48" t="inlineStr"/>
-      <c r="E48" t="inlineStr"/>
-      <c r="F48" t="inlineStr">
-        <is>
-          <t>${q0_9} != 'escola'</t>
-        </is>
-      </c>
-      <c r="G48" t="inlineStr">
-        <is>
-          <t>table-list</t>
-        </is>
-      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr"/>
+      <c r="G48" t="inlineStr"/>
       <c r="H48" t="inlineStr"/>
       <c r="I48" t="inlineStr"/>
       <c r="J48" t="inlineStr"/>
@@ -1750,25 +1758,13 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>select_one qtd_rede_tab</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>q1_1r_01</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>Biblioteca / espaço de leitura</t>
-        </is>
-      </c>
+          <t>end_group</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr"/>
+      <c r="C49" t="inlineStr"/>
       <c r="D49" t="inlineStr"/>
-      <c r="E49" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
+      <c r="E49" t="inlineStr"/>
       <c r="F49" t="inlineStr"/>
       <c r="G49" t="inlineStr"/>
       <c r="H49" t="inlineStr"/>
@@ -1778,27 +1774,31 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>select_one qtd_rede_tab</t>
+          <t>begin_group</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>q1_1r_02</t>
+          <t>t1_1r</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Laboratório de Ciências</t>
+          <t>Q1.1. Infraestrutura da rede — em quantas escolas da rede existe cada espaço?</t>
         </is>
       </c>
       <c r="D50" t="inlineStr"/>
-      <c r="E50" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="F50" t="inlineStr"/>
-      <c r="G50" t="inlineStr"/>
+      <c r="E50" t="inlineStr"/>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>${q0_9} != 'escola'</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>table-list</t>
+        </is>
+      </c>
       <c r="H50" t="inlineStr"/>
       <c r="I50" t="inlineStr"/>
       <c r="J50" t="inlineStr"/>
@@ -1811,12 +1811,12 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>q1_1r_03</t>
+          <t>q1_1r_01</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Laboratório de informática</t>
+          <t>Biblioteca / espaço de leitura</t>
         </is>
       </c>
       <c r="D51" t="inlineStr"/>
@@ -1839,12 +1839,12 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>q1_1r_04</t>
+          <t>q1_1r_02</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Internet</t>
+          <t>Laboratório de Ciências</t>
         </is>
       </c>
       <c r="D52" t="inlineStr"/>
@@ -1867,12 +1867,12 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>q1_1r_05</t>
+          <t>q1_1r_03</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Pátio</t>
+          <t>Laboratório de informática</t>
         </is>
       </c>
       <c r="D53" t="inlineStr"/>
@@ -1895,12 +1895,12 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>q1_1r_06</t>
+          <t>q1_1r_04</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Espaços esportivos</t>
+          <t>Internet</t>
         </is>
       </c>
       <c r="D54" t="inlineStr"/>
@@ -1923,12 +1923,12 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>q1_1r_07</t>
+          <t>q1_1r_05</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Áreas verdes</t>
+          <t>Pátio</t>
         </is>
       </c>
       <c r="D55" t="inlineStr"/>
@@ -1951,12 +1951,12 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>q1_1r_08</t>
+          <t>q1_1r_06</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Horta</t>
+          <t>Espaços esportivos</t>
         </is>
       </c>
       <c r="D56" t="inlineStr"/>
@@ -1979,12 +1979,12 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>q1_1r_09</t>
+          <t>q1_1r_07</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Pomar</t>
+          <t>Áreas verdes</t>
         </is>
       </c>
       <c r="D57" t="inlineStr"/>
@@ -2007,12 +2007,12 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>q1_1r_10</t>
+          <t>q1_1r_08</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Sombreamento</t>
+          <t>Horta</t>
         </is>
       </c>
       <c r="D58" t="inlineStr"/>
@@ -2035,12 +2035,12 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>q1_1r_11</t>
+          <t>q1_1r_09</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Espaços externos para atividades</t>
+          <t>Pomar</t>
         </is>
       </c>
       <c r="D59" t="inlineStr"/>
@@ -2058,13 +2058,25 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>end_group</t>
-        </is>
-      </c>
-      <c r="B60" t="inlineStr"/>
-      <c r="C60" t="inlineStr"/>
+          <t>select_one qtd_rede_tab</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>q1_1r_10</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Sombreamento</t>
+        </is>
+      </c>
       <c r="D60" t="inlineStr"/>
-      <c r="E60" t="inlineStr"/>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
       <c r="F60" t="inlineStr"/>
       <c r="G60" t="inlineStr"/>
       <c r="H60" t="inlineStr"/>
@@ -2074,27 +2086,27 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>select_one qtd_rede_tab</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>q1_2</t>
+          <t>q1_1r_11</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Q1.2. Outra estrutura relevante não listada (se houver)</t>
+          <t>Espaços externos para atividades</t>
         </is>
       </c>
       <c r="D61" t="inlineStr"/>
-      <c r="E61" t="inlineStr"/>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
       <c r="F61" t="inlineStr"/>
-      <c r="G61" t="inlineStr">
-        <is>
-          <t>multiline</t>
-        </is>
-      </c>
+      <c r="G61" t="inlineStr"/>
       <c r="H61" t="inlineStr"/>
       <c r="I61" t="inlineStr"/>
       <c r="J61" t="inlineStr"/>
@@ -2102,30 +2114,26 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>select_multiple termica</t>
+          <t>select_one qtd_rede_tab</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>q1_3</t>
+          <t>q1_1r_12</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Q1.3. Condição térmica das salas de aula</t>
-        </is>
-      </c>
-      <c r="D62" t="inlineStr">
-        <is>
-          <t>A condição térmica costuma variar ao longo do ano — marque todas as situações que se aplicam (ex.: pode ser muito quente no verão E muito fria no inverno).</t>
-        </is>
-      </c>
-      <c r="E62" t="inlineStr"/>
-      <c r="F62" t="inlineStr">
-        <is>
-          <t>${q0_9}='escola'</t>
-        </is>
-      </c>
+          <t>Ar-condicionado nas salas de aula</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr"/>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr"/>
       <c r="G62" t="inlineStr"/>
       <c r="H62" t="inlineStr"/>
       <c r="I62" t="inlineStr"/>
@@ -2134,26 +2142,26 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>select_multiple prob_estrut</t>
+          <t>select_one qtd_rede_tab</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>q1_4</t>
+          <t>q1_1r_13</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Q1.4. Problemas relacionados às condições térmicas/estruturais</t>
+          <t>Ventiladores/estufas nas salas de aula</t>
         </is>
       </c>
       <c r="D63" t="inlineStr"/>
-      <c r="E63" t="inlineStr"/>
-      <c r="F63" t="inlineStr">
-        <is>
-          <t>${q0_9}='escola'</t>
-        </is>
-      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr"/>
       <c r="G63" t="inlineStr"/>
       <c r="H63" t="inlineStr"/>
       <c r="I63" t="inlineStr"/>
@@ -2162,26 +2170,14 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="B64" t="inlineStr">
-        <is>
-          <t>q1_4_outro</t>
-        </is>
-      </c>
-      <c r="C64" t="inlineStr">
-        <is>
-          <t>Especifique (Outro)</t>
-        </is>
-      </c>
+          <t>end_group</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr"/>
+      <c r="C64" t="inlineStr"/>
       <c r="D64" t="inlineStr"/>
       <c r="E64" t="inlineStr"/>
-      <c r="F64" t="inlineStr">
-        <is>
-          <t>(${q0_9}='escola') and selected(${q1_4}, 'outro')</t>
-        </is>
-      </c>
+      <c r="F64" t="inlineStr"/>
       <c r="G64" t="inlineStr"/>
       <c r="H64" t="inlineStr"/>
       <c r="I64" t="inlineStr"/>
@@ -2190,27 +2186,27 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>begin_group</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>e1_escola</t>
+          <t>q1_2</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Água, esgoto e resíduos — escola</t>
+          <t>Q1.2. Outra estrutura relevante não listada (se houver)</t>
         </is>
       </c>
       <c r="D65" t="inlineStr"/>
       <c r="E65" t="inlineStr"/>
-      <c r="F65" t="inlineStr">
-        <is>
-          <t>${q0_9}='escola'</t>
-        </is>
-      </c>
-      <c r="G65" t="inlineStr"/>
+      <c r="F65" t="inlineStr"/>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>multiline</t>
+        </is>
+      </c>
       <c r="H65" t="inlineStr"/>
       <c r="I65" t="inlineStr"/>
       <c r="J65" t="inlineStr"/>
@@ -2218,22 +2214,30 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>select_multiple agua_fonte</t>
+          <t>select_multiple termica</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>q1_5</t>
+          <t>q1_3</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Q1.5. Fonte de abastecimento de água</t>
-        </is>
-      </c>
-      <c r="D66" t="inlineStr"/>
+          <t>Q1.3. Condição térmica das salas de aula</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>A condição térmica costuma variar ao longo do ano — marque todas as situações que se aplicam (ex.: pode ser muito quente no verão E muito fria no inverno).</t>
+        </is>
+      </c>
       <c r="E66" t="inlineStr"/>
-      <c r="F66" t="inlineStr"/>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>${q0_9}='escola'</t>
+        </is>
+      </c>
       <c r="G66" t="inlineStr"/>
       <c r="H66" t="inlineStr"/>
       <c r="I66" t="inlineStr"/>
@@ -2242,24 +2246,24 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>select_multiple prob_estrut</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>q1_5_outro</t>
+          <t>q1_4</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Especifique (Outro)</t>
+          <t>Q1.4. Problemas relacionados às condições térmicas/estruturais</t>
         </is>
       </c>
       <c r="D67" t="inlineStr"/>
       <c r="E67" t="inlineStr"/>
       <c r="F67" t="inlineStr">
         <is>
-          <t>selected(${q1_5}, 'outro')</t>
+          <t>${q0_9}='escola'</t>
         </is>
       </c>
       <c r="G67" t="inlineStr"/>
@@ -2270,22 +2274,26 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>select_one sim_nao_ns</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>q1_6</t>
+          <t>q1_4_outro</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Q1.6. Há interrupções no abastecimento de água?</t>
+          <t>Especifique (Outro)</t>
         </is>
       </c>
       <c r="D68" t="inlineStr"/>
       <c r="E68" t="inlineStr"/>
-      <c r="F68" t="inlineStr"/>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>(${q0_9}='escola') and selected(${q1_4}, 'outro')</t>
+        </is>
+      </c>
       <c r="G68" t="inlineStr"/>
       <c r="H68" t="inlineStr"/>
       <c r="I68" t="inlineStr"/>
@@ -2294,31 +2302,27 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>begin_group</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>q1_7</t>
+          <t>e1_escola</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Q1.7. Em que período(s) isso costuma ocorrer?</t>
+          <t>Água, esgoto e resíduos — escola</t>
         </is>
       </c>
       <c r="D69" t="inlineStr"/>
       <c r="E69" t="inlineStr"/>
       <c r="F69" t="inlineStr">
         <is>
-          <t>${q1_6}='sim'</t>
-        </is>
-      </c>
-      <c r="G69" t="inlineStr">
-        <is>
-          <t>multiline</t>
-        </is>
-      </c>
+          <t>${q0_9}='escola'</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr"/>
       <c r="H69" t="inlineStr"/>
       <c r="I69" t="inlineStr"/>
       <c r="J69" t="inlineStr"/>
@@ -2326,17 +2330,17 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>select_one sim_nao_ns</t>
+          <t>select_multiple agua_fonte</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>q1_8</t>
+          <t>q1_5</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Q1.8. Existe monitoramento da qualidade da água?</t>
+          <t>Q1.5. Fonte de abastecimento de água</t>
         </is>
       </c>
       <c r="D70" t="inlineStr"/>
@@ -2355,26 +2359,22 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>q1_9</t>
+          <t>q1_5_outro</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Q1.9. Quem é responsável por esse monitoramento?</t>
+          <t>Especifique (Outro)</t>
         </is>
       </c>
       <c r="D71" t="inlineStr"/>
       <c r="E71" t="inlineStr"/>
       <c r="F71" t="inlineStr">
         <is>
-          <t>${q1_8}='sim'</t>
-        </is>
-      </c>
-      <c r="G71" t="inlineStr">
-        <is>
-          <t>multiline</t>
-        </is>
-      </c>
+          <t>selected(${q1_5}, 'outro')</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr"/>
       <c r="H71" t="inlineStr"/>
       <c r="I71" t="inlineStr"/>
       <c r="J71" t="inlineStr"/>
@@ -2387,21 +2387,17 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>q1_10</t>
+          <t>q1_6</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Q1.10. Existem registros desse monitoramento?</t>
+          <t>Q1.6. Há interrupções no abastecimento de água?</t>
         </is>
       </c>
       <c r="D72" t="inlineStr"/>
       <c r="E72" t="inlineStr"/>
-      <c r="F72" t="inlineStr">
-        <is>
-          <t>${q1_8}='sim'</t>
-        </is>
-      </c>
+      <c r="F72" t="inlineStr"/>
       <c r="G72" t="inlineStr"/>
       <c r="H72" t="inlineStr"/>
       <c r="I72" t="inlineStr"/>
@@ -2410,23 +2406,31 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>select_multiple infra_hidrica</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>q1_11</t>
+          <t>q1_7</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Q1.11. Infraestrutura hídrica disponível</t>
+          <t>Q1.7. Em que período(s) isso costuma ocorrer?</t>
         </is>
       </c>
       <c r="D73" t="inlineStr"/>
       <c r="E73" t="inlineStr"/>
-      <c r="F73" t="inlineStr"/>
-      <c r="G73" t="inlineStr"/>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>${q1_6}='sim'</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>multiline</t>
+        </is>
+      </c>
       <c r="H73" t="inlineStr"/>
       <c r="I73" t="inlineStr"/>
       <c r="J73" t="inlineStr"/>
@@ -2434,26 +2438,22 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>select_one sim_nao_ns</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>q1_11_outro</t>
+          <t>q1_8</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Especifique (Outro)</t>
+          <t>Q1.8. Existe monitoramento da qualidade da água?</t>
         </is>
       </c>
       <c r="D74" t="inlineStr"/>
       <c r="E74" t="inlineStr"/>
-      <c r="F74" t="inlineStr">
-        <is>
-          <t>selected(${q1_11}, 'outro')</t>
-        </is>
-      </c>
+      <c r="F74" t="inlineStr"/>
       <c r="G74" t="inlineStr"/>
       <c r="H74" t="inlineStr"/>
       <c r="I74" t="inlineStr"/>
@@ -2462,23 +2462,31 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>select_multiple esgoto</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>q1_12</t>
+          <t>q1_9</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Q1.12. Destinação do esgoto</t>
+          <t>Q1.9. Quem é responsável por esse monitoramento?</t>
         </is>
       </c>
       <c r="D75" t="inlineStr"/>
       <c r="E75" t="inlineStr"/>
-      <c r="F75" t="inlineStr"/>
-      <c r="G75" t="inlineStr"/>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>${q1_8}='sim'</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>multiline</t>
+        </is>
+      </c>
       <c r="H75" t="inlineStr"/>
       <c r="I75" t="inlineStr"/>
       <c r="J75" t="inlineStr"/>
@@ -2486,24 +2494,24 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>select_one sim_nao_ns</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>q1_12_outro</t>
+          <t>q1_10</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Especifique (Outro)</t>
+          <t>Q1.10. Existem registros desse monitoramento?</t>
         </is>
       </c>
       <c r="D76" t="inlineStr"/>
       <c r="E76" t="inlineStr"/>
       <c r="F76" t="inlineStr">
         <is>
-          <t>selected(${q1_12}, 'outro')</t>
+          <t>${q1_8}='sim'</t>
         </is>
       </c>
       <c r="G76" t="inlineStr"/>
@@ -2514,17 +2522,17 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>select_one sim_nao_ns</t>
+          <t>select_multiple infra_hidrica</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>q1_13</t>
+          <t>q1_11</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Q1.13. Há esgoto a céu aberto no entorno do local?</t>
+          <t>Q1.11. Infraestrutura hídrica disponível</t>
         </is>
       </c>
       <c r="D77" t="inlineStr"/>
@@ -2538,26 +2546,26 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>select_one sim_nao_ns</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>q1_14</t>
+          <t>q1_11_outro</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Q1.14. Ocorrem alagamentos neste local ou no entorno?</t>
+          <t>Especifique (Outro)</t>
         </is>
       </c>
       <c r="D78" t="inlineStr"/>
-      <c r="E78" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="F78" t="inlineStr"/>
+      <c r="E78" t="inlineStr"/>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>selected(${q1_11}, 'outro')</t>
+        </is>
+      </c>
       <c r="G78" t="inlineStr"/>
       <c r="H78" t="inlineStr"/>
       <c r="I78" t="inlineStr"/>
@@ -2566,31 +2574,23 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>select_multiple esgoto</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>q1_15</t>
+          <t>q1_12</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Q1.15. Em que espaços da escola esses alagamentos costumam ocorrer (Ex: apenas na área externa, invadem as salas, etc)?</t>
+          <t>Q1.12. Destinação do esgoto</t>
         </is>
       </c>
       <c r="D79" t="inlineStr"/>
       <c r="E79" t="inlineStr"/>
-      <c r="F79" t="inlineStr">
-        <is>
-          <t>${q1_14}='sim'</t>
-        </is>
-      </c>
-      <c r="G79" t="inlineStr">
-        <is>
-          <t>multiline</t>
-        </is>
-      </c>
+      <c r="F79" t="inlineStr"/>
+      <c r="G79" t="inlineStr"/>
       <c r="H79" t="inlineStr"/>
       <c r="I79" t="inlineStr"/>
       <c r="J79" t="inlineStr"/>
@@ -2598,24 +2598,24 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>select_multiple impacto_alag</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>q1_16</t>
+          <t>q1_12_outro</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Q1.16. Impactos observados nesses episódios</t>
+          <t>Especifique (Outro)</t>
         </is>
       </c>
       <c r="D80" t="inlineStr"/>
       <c r="E80" t="inlineStr"/>
       <c r="F80" t="inlineStr">
         <is>
-          <t>${q1_14}='sim'</t>
+          <t>selected(${q1_12}, 'outro')</t>
         </is>
       </c>
       <c r="G80" t="inlineStr"/>
@@ -2626,26 +2626,22 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>select_one sim_nao_ns</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>q1_16_outro</t>
+          <t>q1_13</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Especifique (Outro)</t>
+          <t>Q1.13. Há esgoto a céu aberto no entorno do local?</t>
         </is>
       </c>
       <c r="D81" t="inlineStr"/>
       <c r="E81" t="inlineStr"/>
-      <c r="F81" t="inlineStr">
-        <is>
-          <t>(${q1_14}='sim') and selected(${q1_16}, 'outro')</t>
-        </is>
-      </c>
+      <c r="F81" t="inlineStr"/>
       <c r="G81" t="inlineStr"/>
       <c r="H81" t="inlineStr"/>
       <c r="I81" t="inlineStr"/>
@@ -2659,16 +2655,20 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>q1_17</t>
+          <t>q1_14</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Q1.17. Há separação de resíduos neste local?</t>
+          <t>Q1.14. Ocorrem alagamentos neste local ou no entorno?</t>
         </is>
       </c>
       <c r="D82" t="inlineStr"/>
-      <c r="E82" t="inlineStr"/>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
       <c r="F82" t="inlineStr"/>
       <c r="G82" t="inlineStr"/>
       <c r="H82" t="inlineStr"/>
@@ -2678,23 +2678,31 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>select_multiple destino_res</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>q1_18</t>
+          <t>q1_15</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Q1.18. Destinação dos resíduos</t>
+          <t>Q1.15. Em que espaços da escola esses alagamentos costumam ocorrer (Ex: apenas na área externa, invadem as salas, etc)?</t>
         </is>
       </c>
       <c r="D83" t="inlineStr"/>
       <c r="E83" t="inlineStr"/>
-      <c r="F83" t="inlineStr"/>
-      <c r="G83" t="inlineStr"/>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>${q1_14}='sim'</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>multiline</t>
+        </is>
+      </c>
       <c r="H83" t="inlineStr"/>
       <c r="I83" t="inlineStr"/>
       <c r="J83" t="inlineStr"/>
@@ -2702,24 +2710,24 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>select_multiple impacto_alag</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>q1_18_outro</t>
+          <t>q1_16</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Especifique (Outro)</t>
+          <t>Q1.16. Impactos observados nesses episódios</t>
         </is>
       </c>
       <c r="D84" t="inlineStr"/>
       <c r="E84" t="inlineStr"/>
       <c r="F84" t="inlineStr">
         <is>
-          <t>selected(${q1_18}, 'outro')</t>
+          <t>${q1_14}='sim'</t>
         </is>
       </c>
       <c r="G84" t="inlineStr"/>
@@ -2730,62 +2738,50 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>select_multiple prob_res</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>q1_19</t>
+          <t>q1_16_outro</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Q1.19. Existem problemas relacionados a resíduos no entorno do local?</t>
-        </is>
-      </c>
-      <c r="D85" t="inlineStr">
-        <is>
-          <t>Considere a área imediatamente ao redor do local, não o município inteiro.</t>
-        </is>
-      </c>
+          <t>Especifique (Outro)</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr"/>
       <c r="E85" t="inlineStr"/>
-      <c r="F85" t="inlineStr"/>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>(${q1_14}='sim') and selected(${q1_16}, 'outro')</t>
+        </is>
+      </c>
       <c r="G85" t="inlineStr"/>
-      <c r="H85" t="inlineStr">
-        <is>
-          <t>not((selected(., 'nenhum') or selected(., 'nao_sabe')) and count-selected(.) &gt; 1)</t>
-        </is>
-      </c>
-      <c r="I85" t="inlineStr">
-        <is>
-          <t>"Nenhum" e "Não sabe" não podem ser combinados com outras opções.</t>
-        </is>
-      </c>
+      <c r="H85" t="inlineStr"/>
+      <c r="I85" t="inlineStr"/>
       <c r="J85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>select_one sim_nao_ns</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>q1_19_outro</t>
+          <t>q1_17</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Especifique (Outro)</t>
+          <t>Q1.17. Há separação de resíduos neste local?</t>
         </is>
       </c>
       <c r="D86" t="inlineStr"/>
       <c r="E86" t="inlineStr"/>
-      <c r="F86" t="inlineStr">
-        <is>
-          <t>selected(${q1_19}, 'outro')</t>
-        </is>
-      </c>
+      <c r="F86" t="inlineStr"/>
       <c r="G86" t="inlineStr"/>
       <c r="H86" t="inlineStr"/>
       <c r="I86" t="inlineStr"/>
@@ -2794,31 +2790,23 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>select_multiple destino_res</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>q1_20</t>
+          <t>q1_18</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Q1.20. Descreva os problemas causados pela disposição incorreta dos resíduos, caso ocorra.</t>
+          <t>Q1.18. Destinação dos resíduos</t>
         </is>
       </c>
       <c r="D87" t="inlineStr"/>
       <c r="E87" t="inlineStr"/>
-      <c r="F87" t="inlineStr">
-        <is>
-          <t>${q1_19} != '' and not(selected(${q1_19}, 'nenhum')) and not(selected(${q1_19}, 'nao_sabe'))</t>
-        </is>
-      </c>
-      <c r="G87" t="inlineStr">
-        <is>
-          <t>multiline</t>
-        </is>
-      </c>
+      <c r="F87" t="inlineStr"/>
+      <c r="G87" t="inlineStr"/>
       <c r="H87" t="inlineStr"/>
       <c r="I87" t="inlineStr"/>
       <c r="J87" t="inlineStr"/>
@@ -2826,14 +2814,26 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>end_group</t>
-        </is>
-      </c>
-      <c r="B88" t="inlineStr"/>
-      <c r="C88" t="inlineStr"/>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>q1_18_outro</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>Especifique (Outro)</t>
+        </is>
+      </c>
       <c r="D88" t="inlineStr"/>
       <c r="E88" t="inlineStr"/>
-      <c r="F88" t="inlineStr"/>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>selected(${q1_18}, 'outro')</t>
+        </is>
+      </c>
       <c r="G88" t="inlineStr"/>
       <c r="H88" t="inlineStr"/>
       <c r="I88" t="inlineStr"/>
@@ -2842,50 +2842,62 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>begin_group</t>
+          <t>select_multiple prob_res</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>e1_rede</t>
+          <t>q1_19</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Água, esgoto e resíduos — escolas da rede</t>
-        </is>
-      </c>
-      <c r="D89" t="inlineStr"/>
+          <t>Q1.19. Existem problemas relacionados a resíduos no entorno do local?</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>Considere a área imediatamente ao redor do local, não o município inteiro.</t>
+        </is>
+      </c>
       <c r="E89" t="inlineStr"/>
-      <c r="F89" t="inlineStr">
-        <is>
-          <t>${q0_9} != 'escola'</t>
-        </is>
-      </c>
+      <c r="F89" t="inlineStr"/>
       <c r="G89" t="inlineStr"/>
-      <c r="H89" t="inlineStr"/>
-      <c r="I89" t="inlineStr"/>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>not((selected(., 'nenhum') or selected(., 'nao_sabe')) and count-selected(.) &gt; 1)</t>
+        </is>
+      </c>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>"Nenhum" e "Não sabe" não podem ser combinados com outras opções.</t>
+        </is>
+      </c>
       <c r="J89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>e1_rede_nota</t>
+          <t>q1_19_outro</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Responda com base na sua visão geral das escolas da rede/região de atuação. Estimativas são bem-vindas; "Não sabe" é uma resposta válida e vira lacuna de conhecimento registrada.</t>
+          <t>Especifique (Outro)</t>
         </is>
       </c>
       <c r="D90" t="inlineStr"/>
       <c r="E90" t="inlineStr"/>
-      <c r="F90" t="inlineStr"/>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>selected(${q1_19}, 'outro')</t>
+        </is>
+      </c>
       <c r="G90" t="inlineStr"/>
       <c r="H90" t="inlineStr"/>
       <c r="I90" t="inlineStr"/>
@@ -2894,27 +2906,31 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>select_multiple termica</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>q1_3r</t>
+          <t>q1_20</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Q1.3. Condição térmica das salas de aula nas escolas da rede</t>
-        </is>
-      </c>
-      <c r="D91" t="inlineStr">
-        <is>
-          <t>Marque todas as situações que se aplicam à rede.</t>
-        </is>
-      </c>
+          <t>Q1.20. Descreva os problemas causados pela disposição incorreta dos resíduos, caso ocorra.</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr"/>
       <c r="E91" t="inlineStr"/>
-      <c r="F91" t="inlineStr"/>
-      <c r="G91" t="inlineStr"/>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>${q1_19} != '' and not(selected(${q1_19}, 'nenhum')) and not(selected(${q1_19}, 'nao_sabe'))</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>multiline</t>
+        </is>
+      </c>
       <c r="H91" t="inlineStr"/>
       <c r="I91" t="inlineStr"/>
       <c r="J91" t="inlineStr"/>
@@ -2922,19 +2938,11 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>select_multiple prob_estrut</t>
-        </is>
-      </c>
-      <c r="B92" t="inlineStr">
-        <is>
-          <t>q1_4r</t>
-        </is>
-      </c>
-      <c r="C92" t="inlineStr">
-        <is>
-          <t>Q1.4. Problemas estruturais mais comuns nas escolas da rede</t>
-        </is>
-      </c>
+          <t>end_group</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr"/>
+      <c r="C92" t="inlineStr"/>
       <c r="D92" t="inlineStr"/>
       <c r="E92" t="inlineStr"/>
       <c r="F92" t="inlineStr"/>
@@ -2946,24 +2954,24 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>begin_group</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>q1_4r_outro</t>
+          <t>e1_rede</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Especifique (Outro)</t>
+          <t>Água, esgoto e resíduos — escolas da rede</t>
         </is>
       </c>
       <c r="D93" t="inlineStr"/>
       <c r="E93" t="inlineStr"/>
       <c r="F93" t="inlineStr">
         <is>
-          <t>selected(${q1_4r}, 'outro')</t>
+          <t>${q0_9} != 'escola'</t>
         </is>
       </c>
       <c r="G93" t="inlineStr"/>
@@ -2974,25 +2982,21 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>select_multiple agua_fonte</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>q1_5r</t>
+          <t>e1_rede_nota</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Q1.5. Fontes de abastecimento de água das escolas da rede</t>
+          <t>Responda com base na sua visão geral das escolas da rede/região de atuação. Estimativas são bem-vindas; "Não sabe" é uma resposta válida e vira lacuna de conhecimento registrada.</t>
         </is>
       </c>
       <c r="D94" t="inlineStr"/>
-      <c r="E94" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
+      <c r="E94" t="inlineStr"/>
       <c r="F94" t="inlineStr"/>
       <c r="G94" t="inlineStr"/>
       <c r="H94" t="inlineStr"/>
@@ -3002,26 +3006,26 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>select_multiple termica</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>q1_5r_outro</t>
+          <t>q1_3r</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Especifique (Outro)</t>
-        </is>
-      </c>
-      <c r="D95" t="inlineStr"/>
+          <t>Q1.3. Condição térmica das salas de aula nas escolas da rede</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>Marque todas as situações que se aplicam à rede.</t>
+        </is>
+      </c>
       <c r="E95" t="inlineStr"/>
-      <c r="F95" t="inlineStr">
-        <is>
-          <t>selected(${q1_5r}, 'outro')</t>
-        </is>
-      </c>
+      <c r="F95" t="inlineStr"/>
       <c r="G95" t="inlineStr"/>
       <c r="H95" t="inlineStr"/>
       <c r="I95" t="inlineStr"/>
@@ -3030,17 +3034,17 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>select_one qtd_rede</t>
+          <t>select_multiple prob_estrut</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>q1_6r</t>
+          <t>q1_4r</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Q1.6. Em quantas escolas da rede há interrupções no abastecimento de água?</t>
+          <t>Q1.4. Problemas estruturais mais comuns nas escolas da rede</t>
         </is>
       </c>
       <c r="D96" t="inlineStr"/>
@@ -3059,26 +3063,22 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>q1_7r</t>
+          <t>q1_4r_outro</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Q1.7. Em que período(s) isso costuma ocorrer?</t>
+          <t>Especifique (Outro)</t>
         </is>
       </c>
       <c r="D97" t="inlineStr"/>
       <c r="E97" t="inlineStr"/>
       <c r="F97" t="inlineStr">
         <is>
-          <t>${q1_6r} != '' and ${q1_6r} != 'em_nenhuma' and ${q1_6r} != 'nao_sabe'</t>
-        </is>
-      </c>
-      <c r="G97" t="inlineStr">
-        <is>
-          <t>multiline</t>
-        </is>
-      </c>
+          <t>selected(${q1_4r}, 'outro')</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr"/>
       <c r="H97" t="inlineStr"/>
       <c r="I97" t="inlineStr"/>
       <c r="J97" t="inlineStr"/>
@@ -3086,21 +3086,25 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>select_one qtd_rede</t>
+          <t>select_multiple agua_fonte</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>q1_8r</t>
+          <t>q1_5r</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Q1.8. Em quantas escolas da rede há monitoramento da qualidade da água?</t>
+          <t>Q1.5. Fontes de abastecimento de água das escolas da rede</t>
         </is>
       </c>
       <c r="D98" t="inlineStr"/>
-      <c r="E98" t="inlineStr"/>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
       <c r="F98" t="inlineStr"/>
       <c r="G98" t="inlineStr"/>
       <c r="H98" t="inlineStr"/>
@@ -3115,19 +3119,19 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>q1_9r</t>
+          <t>q1_5r_outro</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Q1.9. Quem é responsável por esse monitoramento?</t>
+          <t>Especifique (Outro)</t>
         </is>
       </c>
       <c r="D99" t="inlineStr"/>
       <c r="E99" t="inlineStr"/>
       <c r="F99" t="inlineStr">
         <is>
-          <t>${q1_8r} != '' and ${q1_8r} != 'em_nenhuma' and ${q1_8r} != 'nao_sabe'</t>
+          <t>selected(${q1_5r}, 'outro')</t>
         </is>
       </c>
       <c r="G99" t="inlineStr"/>
@@ -3138,26 +3142,22 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>select_one sim_nao_ns</t>
+          <t>select_one qtd_rede</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>q1_10r</t>
+          <t>q1_6r</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Q1.10. A secretaria/órgão tem acesso aos registros desse monitoramento?</t>
+          <t>Q1.6. Em quantas escolas da rede há interrupções no abastecimento de água?</t>
         </is>
       </c>
       <c r="D100" t="inlineStr"/>
       <c r="E100" t="inlineStr"/>
-      <c r="F100" t="inlineStr">
-        <is>
-          <t>${q1_8r} != '' and ${q1_8r} != 'em_nenhuma' and ${q1_8r} != 'nao_sabe'</t>
-        </is>
-      </c>
+      <c r="F100" t="inlineStr"/>
       <c r="G100" t="inlineStr"/>
       <c r="H100" t="inlineStr"/>
       <c r="I100" t="inlineStr"/>
@@ -3166,23 +3166,31 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>select_multiple infra_hidrica</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>q1_11r</t>
+          <t>q1_7r</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Q1.11. Infraestrutura hídrica presente nas escolas da rede</t>
+          <t>Q1.7. Em que período(s) isso costuma ocorrer?</t>
         </is>
       </c>
       <c r="D101" t="inlineStr"/>
       <c r="E101" t="inlineStr"/>
-      <c r="F101" t="inlineStr"/>
-      <c r="G101" t="inlineStr"/>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>${q1_6r} != '' and ${q1_6r} != 'em_nenhuma' and ${q1_6r} != 'nao_sabe'</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>multiline</t>
+        </is>
+      </c>
       <c r="H101" t="inlineStr"/>
       <c r="I101" t="inlineStr"/>
       <c r="J101" t="inlineStr"/>
@@ -3190,26 +3198,22 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>select_one qtd_rede</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>q1_11r_outro</t>
+          <t>q1_8r</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Especifique (Outro)</t>
+          <t>Q1.8. Em quantas escolas da rede há monitoramento da qualidade da água?</t>
         </is>
       </c>
       <c r="D102" t="inlineStr"/>
       <c r="E102" t="inlineStr"/>
-      <c r="F102" t="inlineStr">
-        <is>
-          <t>selected(${q1_11r}, 'outro')</t>
-        </is>
-      </c>
+      <c r="F102" t="inlineStr"/>
       <c r="G102" t="inlineStr"/>
       <c r="H102" t="inlineStr"/>
       <c r="I102" t="inlineStr"/>
@@ -3218,22 +3222,26 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>select_multiple esgoto</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>q1_12r</t>
+          <t>q1_9r</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Q1.12. Destinação do esgoto nas escolas da rede</t>
+          <t>Q1.9. Quem é responsável por esse monitoramento?</t>
         </is>
       </c>
       <c r="D103" t="inlineStr"/>
       <c r="E103" t="inlineStr"/>
-      <c r="F103" t="inlineStr"/>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>${q1_8r} != '' and ${q1_8r} != 'em_nenhuma' and ${q1_8r} != 'nao_sabe'</t>
+        </is>
+      </c>
       <c r="G103" t="inlineStr"/>
       <c r="H103" t="inlineStr"/>
       <c r="I103" t="inlineStr"/>
@@ -3242,24 +3250,24 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>select_one sim_nao_ns</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>q1_12r_outro</t>
+          <t>q1_10r</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Especifique (Outro)</t>
+          <t>Q1.10. A secretaria/órgão tem acesso aos registros desse monitoramento?</t>
         </is>
       </c>
       <c r="D104" t="inlineStr"/>
       <c r="E104" t="inlineStr"/>
       <c r="F104" t="inlineStr">
         <is>
-          <t>selected(${q1_12r}, 'outro')</t>
+          <t>${q1_8r} != '' and ${q1_8r} != 'em_nenhuma' and ${q1_8r} != 'nao_sabe'</t>
         </is>
       </c>
       <c r="G104" t="inlineStr"/>
@@ -3270,17 +3278,17 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>select_one qtd_rede</t>
+          <t>select_multiple infra_hidrica</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>q1_13r</t>
+          <t>q1_11r</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Q1.13. Em quantas escolas da rede há esgoto a céu aberto no entorno?</t>
+          <t>Q1.11. Infraestrutura hídrica presente nas escolas da rede</t>
         </is>
       </c>
       <c r="D105" t="inlineStr"/>
@@ -3294,26 +3302,26 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>select_one qtd_rede</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>q1_14r</t>
+          <t>q1_11r_outro</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Q1.14. Em quantas escolas da rede ocorrem alagamentos na escola ou no entorno?</t>
+          <t>Especifique (Outro)</t>
         </is>
       </c>
       <c r="D106" t="inlineStr"/>
-      <c r="E106" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="F106" t="inlineStr"/>
+      <c r="E106" t="inlineStr"/>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>selected(${q1_11r}, 'outro')</t>
+        </is>
+      </c>
       <c r="G106" t="inlineStr"/>
       <c r="H106" t="inlineStr"/>
       <c r="I106" t="inlineStr"/>
@@ -3322,31 +3330,23 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>select_multiple esgoto</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>q1_15r</t>
+          <t>q1_12r</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Q1.15. Quais escolas/regiões são mais afetadas?</t>
+          <t>Q1.12. Destinação do esgoto nas escolas da rede</t>
         </is>
       </c>
       <c r="D107" t="inlineStr"/>
       <c r="E107" t="inlineStr"/>
-      <c r="F107" t="inlineStr">
-        <is>
-          <t>${q1_14r} != '' and ${q1_14r} != 'em_nenhuma' and ${q1_14r} != 'nao_sabe'</t>
-        </is>
-      </c>
-      <c r="G107" t="inlineStr">
-        <is>
-          <t>multiline</t>
-        </is>
-      </c>
+      <c r="F107" t="inlineStr"/>
+      <c r="G107" t="inlineStr"/>
       <c r="H107" t="inlineStr"/>
       <c r="I107" t="inlineStr"/>
       <c r="J107" t="inlineStr"/>
@@ -3354,24 +3354,24 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>select_multiple impacto_alag</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>q1_16r</t>
+          <t>q1_12r_outro</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Q1.16. Impactos observados nesses episódios</t>
+          <t>Especifique (Outro)</t>
         </is>
       </c>
       <c r="D108" t="inlineStr"/>
       <c r="E108" t="inlineStr"/>
       <c r="F108" t="inlineStr">
         <is>
-          <t>${q1_14r} != '' and ${q1_14r} != 'em_nenhuma' and ${q1_14r} != 'nao_sabe'</t>
+          <t>selected(${q1_12r}, 'outro')</t>
         </is>
       </c>
       <c r="G108" t="inlineStr"/>
@@ -3382,26 +3382,22 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>select_one qtd_rede</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>q1_16r_outro</t>
+          <t>q1_13r</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Especifique (Outro)</t>
+          <t>Q1.13. Em quantas escolas da rede há esgoto a céu aberto no entorno?</t>
         </is>
       </c>
       <c r="D109" t="inlineStr"/>
       <c r="E109" t="inlineStr"/>
-      <c r="F109" t="inlineStr">
-        <is>
-          <t>(${q1_14r} != '' and ${q1_14r} != 'em_nenhuma' and ${q1_14r} != 'nao_sabe') and selected(${q1_16r}, 'outro')</t>
-        </is>
-      </c>
+      <c r="F109" t="inlineStr"/>
       <c r="G109" t="inlineStr"/>
       <c r="H109" t="inlineStr"/>
       <c r="I109" t="inlineStr"/>
@@ -3415,16 +3411,20 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>q1_17r</t>
+          <t>q1_14r</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>Q1.17. Em quantas escolas da rede há separação de resíduos?</t>
+          <t>Q1.14. Em quantas escolas da rede ocorrem alagamentos na escola ou no entorno?</t>
         </is>
       </c>
       <c r="D110" t="inlineStr"/>
-      <c r="E110" t="inlineStr"/>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
       <c r="F110" t="inlineStr"/>
       <c r="G110" t="inlineStr"/>
       <c r="H110" t="inlineStr"/>
@@ -3434,23 +3434,31 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>select_multiple destino_res</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>q1_18r</t>
+          <t>q1_15r</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Q1.18. Destinação dos resíduos nas escolas da rede</t>
+          <t>Q1.15. Quais escolas/regiões são mais afetadas?</t>
         </is>
       </c>
       <c r="D111" t="inlineStr"/>
       <c r="E111" t="inlineStr"/>
-      <c r="F111" t="inlineStr"/>
-      <c r="G111" t="inlineStr"/>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>${q1_14r} != '' and ${q1_14r} != 'em_nenhuma' and ${q1_14r} != 'nao_sabe'</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>multiline</t>
+        </is>
+      </c>
       <c r="H111" t="inlineStr"/>
       <c r="I111" t="inlineStr"/>
       <c r="J111" t="inlineStr"/>
@@ -3458,24 +3466,24 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>select_multiple impacto_alag</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>q1_18r_outro</t>
+          <t>q1_16r</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>Especifique (Outro)</t>
+          <t>Q1.16. Impactos observados nesses episódios</t>
         </is>
       </c>
       <c r="D112" t="inlineStr"/>
       <c r="E112" t="inlineStr"/>
       <c r="F112" t="inlineStr">
         <is>
-          <t>selected(${q1_18r}, 'outro')</t>
+          <t>${q1_14r} != '' and ${q1_14r} != 'em_nenhuma' and ${q1_14r} != 'nao_sabe'</t>
         </is>
       </c>
       <c r="G112" t="inlineStr"/>
@@ -3486,62 +3494,50 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>select_multiple prob_res</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>q1_19r</t>
+          <t>q1_16r_outro</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Q1.19. Problemas relacionados a resíduos no entorno das escolas da rede</t>
-        </is>
-      </c>
-      <c r="D113" t="inlineStr">
-        <is>
-          <t>Considere a área imediatamente ao redor das escolas, não o município inteiro.</t>
-        </is>
-      </c>
+          <t>Especifique (Outro)</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr"/>
       <c r="E113" t="inlineStr"/>
-      <c r="F113" t="inlineStr"/>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>(${q1_14r} != '' and ${q1_14r} != 'em_nenhuma' and ${q1_14r} != 'nao_sabe') and selected(${q1_16r}, 'outro')</t>
+        </is>
+      </c>
       <c r="G113" t="inlineStr"/>
-      <c r="H113" t="inlineStr">
-        <is>
-          <t>not((selected(., 'nenhum') or selected(., 'nao_sabe')) and count-selected(.) &gt; 1)</t>
-        </is>
-      </c>
-      <c r="I113" t="inlineStr">
-        <is>
-          <t>"Nenhum" e "Não sabe" não podem ser combinados com outras opções.</t>
-        </is>
-      </c>
+      <c r="H113" t="inlineStr"/>
+      <c r="I113" t="inlineStr"/>
       <c r="J113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>select_one qtd_rede</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>q1_19r_outro</t>
+          <t>q1_17r</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>Especifique (Outro)</t>
+          <t>Q1.17. Em quantas escolas da rede há separação de resíduos?</t>
         </is>
       </c>
       <c r="D114" t="inlineStr"/>
       <c r="E114" t="inlineStr"/>
-      <c r="F114" t="inlineStr">
-        <is>
-          <t>selected(${q1_19r}, 'outro')</t>
-        </is>
-      </c>
+      <c r="F114" t="inlineStr"/>
       <c r="G114" t="inlineStr"/>
       <c r="H114" t="inlineStr"/>
       <c r="I114" t="inlineStr"/>
@@ -3550,31 +3546,23 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>select_multiple destino_res</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>q1_20r</t>
+          <t>q1_18r</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>Q1.20. Descreva os problemas causados pela disposição incorreta dos resíduos, caso ocorra.</t>
+          <t>Q1.18. Destinação dos resíduos nas escolas da rede</t>
         </is>
       </c>
       <c r="D115" t="inlineStr"/>
       <c r="E115" t="inlineStr"/>
-      <c r="F115" t="inlineStr">
-        <is>
-          <t>${q1_19r} != '' and not(selected(${q1_19r}, 'nenhum')) and not(selected(${q1_19r}, 'nao_sabe'))</t>
-        </is>
-      </c>
-      <c r="G115" t="inlineStr">
-        <is>
-          <t>multiline</t>
-        </is>
-      </c>
+      <c r="F115" t="inlineStr"/>
+      <c r="G115" t="inlineStr"/>
       <c r="H115" t="inlineStr"/>
       <c r="I115" t="inlineStr"/>
       <c r="J115" t="inlineStr"/>
@@ -3582,14 +3570,26 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>end_group</t>
-        </is>
-      </c>
-      <c r="B116" t="inlineStr"/>
-      <c r="C116" t="inlineStr"/>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>q1_18r_outro</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>Especifique (Outro)</t>
+        </is>
+      </c>
       <c r="D116" t="inlineStr"/>
       <c r="E116" t="inlineStr"/>
-      <c r="F116" t="inlineStr"/>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>selected(${q1_18r}, 'outro')</t>
+        </is>
+      </c>
       <c r="G116" t="inlineStr"/>
       <c r="H116" t="inlineStr"/>
       <c r="I116" t="inlineStr"/>
@@ -3598,33 +3598,37 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>select_multiple elementos</t>
+          <t>select_multiple prob_res</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>q1_21</t>
+          <t>q1_19r</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>Q1.21. Elementos presentes no território de atuação</t>
+          <t>Q1.19. Problemas relacionados a resíduos no entorno das escolas da rede</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>Considere o território mais imediato — para uma local, o bairro ou a região do entorno em que a comunidade escolar circula; para uma secretaria ou regional, a área de abrangência da rede (não o município inteiro, se a atuação for menor). A existência de um elemento não significa, por si só, risco ou impacto, isso será explorado a seguir.</t>
-        </is>
-      </c>
-      <c r="E117" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
+          <t>Considere a área imediatamente ao redor das escolas, não o município inteiro.</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr"/>
       <c r="F117" t="inlineStr"/>
       <c r="G117" t="inlineStr"/>
-      <c r="H117" t="inlineStr"/>
-      <c r="I117" t="inlineStr"/>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>not((selected(., 'nenhum') or selected(., 'nao_sabe')) and count-selected(.) &gt; 1)</t>
+        </is>
+      </c>
+      <c r="I117" t="inlineStr">
+        <is>
+          <t>"Nenhum" e "Não sabe" não podem ser combinados com outras opções.</t>
+        </is>
+      </c>
       <c r="J117" t="inlineStr"/>
     </row>
     <row r="118">
@@ -3635,7 +3639,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>q1_21_outro</t>
+          <t>q1_19r_outro</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
@@ -3647,7 +3651,7 @@
       <c r="E118" t="inlineStr"/>
       <c r="F118" t="inlineStr">
         <is>
-          <t>selected(${q1_21}, 'outro')</t>
+          <t>selected(${q1_19r}, 'outro')</t>
         </is>
       </c>
       <c r="G118" t="inlineStr"/>
@@ -3658,29 +3662,29 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>begin_group</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>t1_22</t>
+          <t>q1_20r</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>Q1.22. Para cada elemento selecionado, qual sua relação com o local/comunidade?</t>
+          <t>Q1.20. Descreva os problemas causados pela disposição incorreta dos resíduos, caso ocorra.</t>
         </is>
       </c>
       <c r="D119" t="inlineStr"/>
       <c r="E119" t="inlineStr"/>
       <c r="F119" t="inlineStr">
         <is>
-          <t>${q1_21} != ''</t>
+          <t>${q1_19r} != '' and not(selected(${q1_19r}, 'nenhum')) and not(selected(${q1_19r}, 'nao_sabe'))</t>
         </is>
       </c>
       <c r="G119" t="inlineStr">
         <is>
-          <t>table-list</t>
+          <t>multiline</t>
         </is>
       </c>
       <c r="H119" t="inlineStr"/>
@@ -3690,26 +3694,14 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>select_multiple relacao_elem</t>
-        </is>
-      </c>
-      <c r="B120" t="inlineStr">
-        <is>
-          <t>q1_22_01</t>
-        </is>
-      </c>
-      <c r="C120" t="inlineStr">
-        <is>
-          <t>Rios/córregos</t>
-        </is>
-      </c>
+          <t>end_group</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr"/>
+      <c r="C120" t="inlineStr"/>
       <c r="D120" t="inlineStr"/>
       <c r="E120" t="inlineStr"/>
-      <c r="F120" t="inlineStr">
-        <is>
-          <t>selected(${q1_21}, 'rios_corregos')</t>
-        </is>
-      </c>
+      <c r="F120" t="inlineStr"/>
       <c r="G120" t="inlineStr"/>
       <c r="H120" t="inlineStr"/>
       <c r="I120" t="inlineStr"/>
@@ -3718,26 +3710,30 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>select_multiple relacao_elem</t>
+          <t>select_multiple elementos</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>q1_22_02</t>
+          <t>q1_21</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>Lagoas/lagos/reservatórios</t>
-        </is>
-      </c>
-      <c r="D121" t="inlineStr"/>
-      <c r="E121" t="inlineStr"/>
-      <c r="F121" t="inlineStr">
-        <is>
-          <t>selected(${q1_21}, 'lagoas_lagos_reservatorios')</t>
-        </is>
-      </c>
+          <t>Q1.21. Elementos presentes no território de atuação</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>Considere o território mais imediato — para uma local, o bairro ou a região do entorno em que a comunidade escolar circula; para uma secretaria ou regional, a área de abrangência da rede (não o município inteiro, se a atuação for menor). A existência de um elemento não significa, por si só, risco ou impacto, isso será explorado a seguir.</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr"/>
       <c r="G121" t="inlineStr"/>
       <c r="H121" t="inlineStr"/>
       <c r="I121" t="inlineStr"/>
@@ -3746,24 +3742,24 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>select_multiple relacao_elem</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>q1_22_03</t>
+          <t>q1_21_outro</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>Áreas de vegetação nativa (matas, florestas, campos)</t>
+          <t>Especifique (Outro)</t>
         </is>
       </c>
       <c r="D122" t="inlineStr"/>
       <c r="E122" t="inlineStr"/>
       <c r="F122" t="inlineStr">
         <is>
-          <t>selected(${q1_21}, 'areas_de_vegetacao_nativa')</t>
+          <t>selected(${q1_21}, 'outro')</t>
         </is>
       </c>
       <c r="G122" t="inlineStr"/>
@@ -3774,27 +3770,31 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>select_multiple relacao_elem</t>
+          <t>begin_group</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>q1_22_04</t>
+          <t>t1_22</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>Parques</t>
+          <t>Q1.22. Para cada elemento selecionado, qual sua relação com o local/comunidade?</t>
         </is>
       </c>
       <c r="D123" t="inlineStr"/>
       <c r="E123" t="inlineStr"/>
       <c r="F123" t="inlineStr">
         <is>
-          <t>selected(${q1_21}, 'parques')</t>
-        </is>
-      </c>
-      <c r="G123" t="inlineStr"/>
+          <t>${q1_21} != ''</t>
+        </is>
+      </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>table-list</t>
+        </is>
+      </c>
       <c r="H123" t="inlineStr"/>
       <c r="I123" t="inlineStr"/>
       <c r="J123" t="inlineStr"/>
@@ -3807,19 +3807,19 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>q1_22_05</t>
+          <t>q1_22_01</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>Encostas</t>
+          <t>Rios/córregos</t>
         </is>
       </c>
       <c r="D124" t="inlineStr"/>
       <c r="E124" t="inlineStr"/>
       <c r="F124" t="inlineStr">
         <is>
-          <t>selected(${q1_21}, 'encostas')</t>
+          <t>selected(${q1_21}, 'rios_corregos')</t>
         </is>
       </c>
       <c r="G124" t="inlineStr"/>
@@ -3835,19 +3835,19 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>q1_22_06</t>
+          <t>q1_22_02</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>Agricultura</t>
+          <t>Lagoas/lagos/reservatórios</t>
         </is>
       </c>
       <c r="D125" t="inlineStr"/>
       <c r="E125" t="inlineStr"/>
       <c r="F125" t="inlineStr">
         <is>
-          <t>selected(${q1_21}, 'agricultura')</t>
+          <t>selected(${q1_21}, 'lagoas_lagos_reservatorios')</t>
         </is>
       </c>
       <c r="G125" t="inlineStr"/>
@@ -3863,19 +3863,19 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>q1_22_07</t>
+          <t>q1_22_03</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>Indústria</t>
+          <t>Áreas de vegetação nativa (matas, florestas, campos)</t>
         </is>
       </c>
       <c r="D126" t="inlineStr"/>
       <c r="E126" t="inlineStr"/>
       <c r="F126" t="inlineStr">
         <is>
-          <t>selected(${q1_21}, 'industria')</t>
+          <t>selected(${q1_21}, 'areas_de_vegetacao_nativa')</t>
         </is>
       </c>
       <c r="G126" t="inlineStr"/>
@@ -3891,19 +3891,19 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>q1_22_08</t>
+          <t>q1_22_04</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>Mineração</t>
+          <t>Parques</t>
         </is>
       </c>
       <c r="D127" t="inlineStr"/>
       <c r="E127" t="inlineStr"/>
       <c r="F127" t="inlineStr">
         <is>
-          <t>selected(${q1_21}, 'mineracao')</t>
+          <t>selected(${q1_21}, 'parques')</t>
         </is>
       </c>
       <c r="G127" t="inlineStr"/>
@@ -3919,19 +3919,19 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>q1_22_09</t>
+          <t>q1_22_05</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>Aterro/lixão</t>
+          <t>Encostas</t>
         </is>
       </c>
       <c r="D128" t="inlineStr"/>
       <c r="E128" t="inlineStr"/>
       <c r="F128" t="inlineStr">
         <is>
-          <t>selected(${q1_21}, 'aterro_lixao')</t>
+          <t>selected(${q1_21}, 'encostas')</t>
         </is>
       </c>
       <c r="G128" t="inlineStr"/>
@@ -3947,19 +3947,19 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>q1_22_10</t>
+          <t>q1_22_06</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>Áreas queimadas</t>
+          <t>Agricultura</t>
         </is>
       </c>
       <c r="D129" t="inlineStr"/>
       <c r="E129" t="inlineStr"/>
       <c r="F129" t="inlineStr">
         <is>
-          <t>selected(${q1_21}, 'areas_queimadas')</t>
+          <t>selected(${q1_21}, 'agricultura')</t>
         </is>
       </c>
       <c r="G129" t="inlineStr"/>
@@ -3975,19 +3975,19 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>q1_22_11</t>
+          <t>q1_22_07</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>Áreas inundáveis</t>
+          <t>Indústria</t>
         </is>
       </c>
       <c r="D130" t="inlineStr"/>
       <c r="E130" t="inlineStr"/>
       <c r="F130" t="inlineStr">
         <is>
-          <t>selected(${q1_21}, 'areas_inundaveis')</t>
+          <t>selected(${q1_21}, 'industria')</t>
         </is>
       </c>
       <c r="G130" t="inlineStr"/>
@@ -4003,19 +4003,19 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>q1_22_12</t>
+          <t>q1_22_08</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>Comércios</t>
+          <t>Mineração</t>
         </is>
       </c>
       <c r="D131" t="inlineStr"/>
       <c r="E131" t="inlineStr"/>
       <c r="F131" t="inlineStr">
         <is>
-          <t>selected(${q1_21}, 'comercios')</t>
+          <t>selected(${q1_21}, 'mineracao')</t>
         </is>
       </c>
       <c r="G131" t="inlineStr"/>
@@ -4031,19 +4031,19 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>q1_22_13</t>
+          <t>q1_22_09</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>Outras áreas degradadas</t>
+          <t>Aterro/lixão</t>
         </is>
       </c>
       <c r="D132" t="inlineStr"/>
       <c r="E132" t="inlineStr"/>
       <c r="F132" t="inlineStr">
         <is>
-          <t>selected(${q1_21}, 'outras_areas_degradadas')</t>
+          <t>selected(${q1_21}, 'aterro_lixao')</t>
         </is>
       </c>
       <c r="G132" t="inlineStr"/>
@@ -4059,19 +4059,19 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>q1_22_14</t>
+          <t>q1_22_10</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>Equipamentos Urbanos</t>
+          <t>Áreas queimadas</t>
         </is>
       </c>
       <c r="D133" t="inlineStr"/>
       <c r="E133" t="inlineStr"/>
       <c r="F133" t="inlineStr">
         <is>
-          <t>selected(${q1_21}, 'equipamentos_urbanos')</t>
+          <t>selected(${q1_21}, 'areas_queimadas')</t>
         </is>
       </c>
       <c r="G133" t="inlineStr"/>
@@ -4087,19 +4087,19 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>q1_22_15</t>
+          <t>q1_22_11</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>Outros</t>
+          <t>Áreas inundáveis</t>
         </is>
       </c>
       <c r="D134" t="inlineStr"/>
       <c r="E134" t="inlineStr"/>
       <c r="F134" t="inlineStr">
         <is>
-          <t>selected(${q1_21}, 'outro')</t>
+          <t>selected(${q1_21}, 'areas_inundaveis')</t>
         </is>
       </c>
       <c r="G134" t="inlineStr"/>
@@ -4110,14 +4110,26 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>end_group</t>
-        </is>
-      </c>
-      <c r="B135" t="inlineStr"/>
-      <c r="C135" t="inlineStr"/>
+          <t>select_multiple relacao_elem</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>q1_22_12</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>Comércios</t>
+        </is>
+      </c>
       <c r="D135" t="inlineStr"/>
       <c r="E135" t="inlineStr"/>
-      <c r="F135" t="inlineStr"/>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>selected(${q1_21}, 'comercios')</t>
+        </is>
+      </c>
       <c r="G135" t="inlineStr"/>
       <c r="H135" t="inlineStr"/>
       <c r="I135" t="inlineStr"/>
@@ -4126,24 +4138,24 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>select_multiple relacao_elem</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>q1_22_nota</t>
+          <t>q1_22_13</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>Nota para tutoria: um mesmo elemento pode ter mais de uma relação ao mesmo tempo (ex.: um rio pode ser, simultaneamente, ambiente e cultura, ou risco e uso comunitário) — marque quantas se aplicarem.</t>
+          <t>Outras áreas degradadas</t>
         </is>
       </c>
       <c r="D136" t="inlineStr"/>
       <c r="E136" t="inlineStr"/>
       <c r="F136" t="inlineStr">
         <is>
-          <t>${q1_21} != ''</t>
+          <t>selected(${q1_21}, 'outras_areas_degradadas')</t>
         </is>
       </c>
       <c r="G136" t="inlineStr"/>
@@ -4154,22 +4166,26 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>select_multiple ativ_econ</t>
+          <t>select_multiple relacao_elem</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>q1_23</t>
+          <t>q1_22_14</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>Q1.23. Principais atividades econômicas do território</t>
+          <t>Equipamentos Urbanos</t>
         </is>
       </c>
       <c r="D137" t="inlineStr"/>
       <c r="E137" t="inlineStr"/>
-      <c r="F137" t="inlineStr"/>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>selected(${q1_21}, 'equipamentos_urbanos')</t>
+        </is>
+      </c>
       <c r="G137" t="inlineStr"/>
       <c r="H137" t="inlineStr"/>
       <c r="I137" t="inlineStr"/>
@@ -4178,24 +4194,24 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>select_multiple relacao_elem</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>q1_23_outro</t>
+          <t>q1_22_15</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>Especifique (Outro)</t>
+          <t>Outros</t>
         </is>
       </c>
       <c r="D138" t="inlineStr"/>
       <c r="E138" t="inlineStr"/>
       <c r="F138" t="inlineStr">
         <is>
-          <t>selected(${q1_23}, 'outro')</t>
+          <t>selected(${q1_21}, 'outro')</t>
         </is>
       </c>
       <c r="G138" t="inlineStr"/>
@@ -4206,19 +4222,11 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>select_one sim_nao_ns</t>
-        </is>
-      </c>
-      <c r="B139" t="inlineStr">
-        <is>
-          <t>q1_24</t>
-        </is>
-      </c>
-      <c r="C139" t="inlineStr">
-        <is>
-          <t>Q1.24. Essas atividades têm impacto percebido no ambiente ou na comunidade (Ex: odor desagradável, excesso de veículos pesados, etc)?</t>
-        </is>
-      </c>
+          <t>end_group</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr"/>
+      <c r="C139" t="inlineStr"/>
       <c r="D139" t="inlineStr"/>
       <c r="E139" t="inlineStr"/>
       <c r="F139" t="inlineStr"/>
@@ -4230,31 +4238,27 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>q1_25</t>
+          <t>q1_22_nota</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>Q1.25. Descreva os impactos percebidos por atividade</t>
+          <t>Nota para tutoria: um mesmo elemento pode ter mais de uma relação ao mesmo tempo (ex.: um rio pode ser, simultaneamente, ambiente e cultura, ou risco e uso comunitário) — marque quantas se aplicarem.</t>
         </is>
       </c>
       <c r="D140" t="inlineStr"/>
       <c r="E140" t="inlineStr"/>
       <c r="F140" t="inlineStr">
         <is>
-          <t>${q1_24}='sim'</t>
-        </is>
-      </c>
-      <c r="G140" t="inlineStr">
-        <is>
-          <t>multiline</t>
-        </is>
-      </c>
+          <t>${q1_21} != ''</t>
+        </is>
+      </c>
+      <c r="G140" t="inlineStr"/>
       <c r="H140" t="inlineStr"/>
       <c r="I140" t="inlineStr"/>
       <c r="J140" t="inlineStr"/>
@@ -4262,17 +4266,17 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>select_one sim_nao_ns</t>
+          <t>select_multiple ativ_econ</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>q1_26</t>
+          <t>q1_23</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>Q1.26. Há eventos sazonais que afetam o local/comunidade (safras, secas, chuvas, festas, etc.)?</t>
+          <t>Q1.23. Principais atividades econômicas do território</t>
         </is>
       </c>
       <c r="D141" t="inlineStr"/>
@@ -4291,26 +4295,22 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>q1_27</t>
+          <t>q1_23_outro</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>Q1.27. Qual é esse evento? Descreva-o, incluindo o período do ano que costuma ocorrer.</t>
+          <t>Especifique (Outro)</t>
         </is>
       </c>
       <c r="D142" t="inlineStr"/>
       <c r="E142" t="inlineStr"/>
       <c r="F142" t="inlineStr">
         <is>
-          <t>${q1_26}='sim'</t>
-        </is>
-      </c>
-      <c r="G142" t="inlineStr">
-        <is>
-          <t>multiline</t>
-        </is>
-      </c>
+          <t>selected(${q1_23}, 'outro')</t>
+        </is>
+      </c>
+      <c r="G142" t="inlineStr"/>
       <c r="H142" t="inlineStr"/>
       <c r="I142" t="inlineStr"/>
       <c r="J142" t="inlineStr"/>
@@ -4318,31 +4318,23 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>select_one sim_nao_ns</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>q1_29</t>
+          <t>q1_24</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>Q1.29. Qual o impacto desse evento neste local?</t>
+          <t>Q1.24. Essas atividades têm impacto percebido no ambiente ou na comunidade (Ex: odor desagradável, excesso de veículos pesados, etc)?</t>
         </is>
       </c>
       <c r="D143" t="inlineStr"/>
       <c r="E143" t="inlineStr"/>
-      <c r="F143" t="inlineStr">
-        <is>
-          <t>${q1_26}='sim'</t>
-        </is>
-      </c>
-      <c r="G143" t="inlineStr">
-        <is>
-          <t>multiline</t>
-        </is>
-      </c>
+      <c r="F143" t="inlineStr"/>
+      <c r="G143" t="inlineStr"/>
       <c r="H143" t="inlineStr"/>
       <c r="I143" t="inlineStr"/>
       <c r="J143" t="inlineStr"/>
@@ -4350,27 +4342,31 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>select_one sim_nao_ns</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>q1_30</t>
+          <t>q1_25</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>Q1.30. Há histórico recente de eventos climáticos extremos que afetaram o local/comunidade?</t>
+          <t>Q1.25. Descreva os impactos percebidos por atividade</t>
         </is>
       </c>
       <c r="D144" t="inlineStr"/>
-      <c r="E144" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="F144" t="inlineStr"/>
-      <c r="G144" t="inlineStr"/>
+      <c r="E144" t="inlineStr"/>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>${q1_24}='sim'</t>
+        </is>
+      </c>
+      <c r="G144" t="inlineStr">
+        <is>
+          <t>multiline</t>
+        </is>
+      </c>
       <c r="H144" t="inlineStr"/>
       <c r="I144" t="inlineStr"/>
       <c r="J144" t="inlineStr"/>
@@ -4378,31 +4374,27 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>select_one sim_nao_ns</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>q1_31</t>
+          <t>q1_26</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>Q1.31. Descreva o(s) evento(s) e a intensidade.</t>
-        </is>
-      </c>
-      <c r="D145" t="inlineStr"/>
+          <t>Q1.26. Há eventos sazonais que afetam o local/comunidade (safras, secas, chuvas, festas, etc.)?</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>Os eventos sazonais podem ter efeitos negativos e/ou positivos.</t>
+        </is>
+      </c>
       <c r="E145" t="inlineStr"/>
-      <c r="F145" t="inlineStr">
-        <is>
-          <t>${q1_30}='sim'</t>
-        </is>
-      </c>
-      <c r="G145" t="inlineStr">
-        <is>
-          <t>multiline</t>
-        </is>
-      </c>
+      <c r="F145" t="inlineStr"/>
+      <c r="G145" t="inlineStr"/>
       <c r="H145" t="inlineStr"/>
       <c r="I145" t="inlineStr"/>
       <c r="J145" t="inlineStr"/>
@@ -4415,22 +4407,26 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>q1_32</t>
+          <t>q1_27</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>Q1.32. Quando ocorreu(ram)?</t>
+          <t>Q1.27. Qual é esse evento? Descreva-o, incluindo o período do ano que costuma ocorrer.</t>
         </is>
       </c>
       <c r="D146" t="inlineStr"/>
       <c r="E146" t="inlineStr"/>
       <c r="F146" t="inlineStr">
         <is>
-          <t>${q1_30}='sim'</t>
-        </is>
-      </c>
-      <c r="G146" t="inlineStr"/>
+          <t>${q1_26}='sim'</t>
+        </is>
+      </c>
+      <c r="G146" t="inlineStr">
+        <is>
+          <t>multiline</t>
+        </is>
+      </c>
       <c r="H146" t="inlineStr"/>
       <c r="I146" t="inlineStr"/>
       <c r="J146" t="inlineStr"/>
@@ -4438,27 +4434,35 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>select_multiple impacto_clima</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>q1_33</t>
+          <t>q1_29</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>Q1.33. Impactos observados</t>
-        </is>
-      </c>
-      <c r="D147" t="inlineStr"/>
+          <t>Q1.29. Qual o impacto desse evento neste local?</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>Os impactos podem ser negativos e/ou positivos (ex.: negativo — falta de água, aulas suspensas; positivo — chuvas que renovam as nascentes, safra que gera renda para as famílias). Descreva ambos, se houver.</t>
+        </is>
+      </c>
       <c r="E147" t="inlineStr"/>
       <c r="F147" t="inlineStr">
         <is>
-          <t>${q1_30}='sim'</t>
-        </is>
-      </c>
-      <c r="G147" t="inlineStr"/>
+          <t>${q1_26}='sim'</t>
+        </is>
+      </c>
+      <c r="G147" t="inlineStr">
+        <is>
+          <t>multiline</t>
+        </is>
+      </c>
       <c r="H147" t="inlineStr"/>
       <c r="I147" t="inlineStr"/>
       <c r="J147" t="inlineStr"/>
@@ -4466,26 +4470,30 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>select_one sim_nao_ns</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>q1_33_outro</t>
+          <t>q1_30</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>Especifique (Outro)</t>
-        </is>
-      </c>
-      <c r="D148" t="inlineStr"/>
-      <c r="E148" t="inlineStr"/>
-      <c r="F148" t="inlineStr">
-        <is>
-          <t>(${q1_30}='sim') and selected(${q1_33}, 'outro')</t>
-        </is>
-      </c>
+          <t>Q1.30. Há histórico recente de eventos climáticos extremos que afetaram o local/comunidade?</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>Eventos climáticos extremos são fenômenos fora do padrão habitual, como ciclones, queimadas, ondas de calor, períodos de seca extrema, enchentes, vendavais, granizo, entre outros.</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="F148" t="inlineStr"/>
       <c r="G148" t="inlineStr"/>
       <c r="H148" t="inlineStr"/>
       <c r="I148" t="inlineStr"/>
@@ -4499,12 +4507,12 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>q1_34</t>
+          <t>q1_31</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>Q1.34. O que o local/comunidade aprendeu com esse evento?</t>
+          <t>Q1.31. Descreva o(s) evento(s) e a intensidade.</t>
         </is>
       </c>
       <c r="D149" t="inlineStr"/>
@@ -4526,22 +4534,26 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>begin_repeat</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>evid_e1</t>
+          <t>q1_32</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>Evidências — Evidências sobre o local e o território</t>
+          <t>Q1.32. Quando ocorreu(ram)?</t>
         </is>
       </c>
       <c r="D150" t="inlineStr"/>
       <c r="E150" t="inlineStr"/>
-      <c r="F150" t="inlineStr"/>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>${q1_30}='sim'</t>
+        </is>
+      </c>
       <c r="G150" t="inlineStr"/>
       <c r="H150" t="inlineStr"/>
       <c r="I150" t="inlineStr"/>
@@ -4550,22 +4562,26 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>select_multiple impacto_clima</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>evid_e1_nota</t>
+          <t>q1_33</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>Evidências sustentam análises futuras (problemas, prioridades, plano de ação). Registrar não é obrigatório para todo campo, mas fortalece a rastreabilidade do diagnóstico.</t>
+          <t>Q1.33. Impactos observados</t>
         </is>
       </c>
       <c r="D151" t="inlineStr"/>
       <c r="E151" t="inlineStr"/>
-      <c r="F151" t="inlineStr"/>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>${q1_30}='sim'</t>
+        </is>
+      </c>
       <c r="G151" t="inlineStr"/>
       <c r="H151" t="inlineStr"/>
       <c r="I151" t="inlineStr"/>
@@ -4574,22 +4590,26 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>select_one tipo_evid</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>evid_e1_tipo</t>
+          <t>q1_33_outro</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>Tipo de evidência</t>
+          <t>Especifique (Outro)</t>
         </is>
       </c>
       <c r="D152" t="inlineStr"/>
       <c r="E152" t="inlineStr"/>
-      <c r="F152" t="inlineStr"/>
+      <c r="F152" t="inlineStr">
+        <is>
+          <t>(${q1_30}='sim') and selected(${q1_33}, 'outro')</t>
+        </is>
+      </c>
       <c r="G152" t="inlineStr"/>
       <c r="H152" t="inlineStr"/>
       <c r="I152" t="inlineStr"/>
@@ -4603,22 +4623,26 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>evid_e1_tipo_outro</t>
+          <t>q1_34</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>Especifique (Outro)</t>
+          <t>Q1.34. O que o local/comunidade aprendeu com esse evento?</t>
         </is>
       </c>
       <c r="D153" t="inlineStr"/>
       <c r="E153" t="inlineStr"/>
       <c r="F153" t="inlineStr">
         <is>
-          <t>${evid_e1_tipo}='outro'</t>
-        </is>
-      </c>
-      <c r="G153" t="inlineStr"/>
+          <t>${q1_30}='sim'</t>
+        </is>
+      </c>
+      <c r="G153" t="inlineStr">
+        <is>
+          <t>multiline</t>
+        </is>
+      </c>
       <c r="H153" t="inlineStr"/>
       <c r="I153" t="inlineStr"/>
       <c r="J153" t="inlineStr"/>
@@ -4626,27 +4650,23 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>begin_repeat</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>evid_e1_desc</t>
+          <t>evid_e1</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>Descreva a evidência</t>
+          <t>Evidências — Evidências sobre o local e o território</t>
         </is>
       </c>
       <c r="D154" t="inlineStr"/>
       <c r="E154" t="inlineStr"/>
       <c r="F154" t="inlineStr"/>
-      <c r="G154" t="inlineStr">
-        <is>
-          <t>multiline</t>
-        </is>
-      </c>
+      <c r="G154" t="inlineStr"/>
       <c r="H154" t="inlineStr"/>
       <c r="I154" t="inlineStr"/>
       <c r="J154" t="inlineStr"/>
@@ -4654,17 +4674,17 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>file</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>evid_e1_anexo</t>
+          <t>evid_e1_nota</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>Anexo (foto/documento) — opcional</t>
+          <t>Evidências sustentam análises futuras (problemas, prioridades, plano de ação). Registrar não é obrigatório para todo campo, mas fortalece a rastreabilidade do diagnóstico.</t>
         </is>
       </c>
       <c r="D155" t="inlineStr"/>
@@ -4678,11 +4698,19 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>end_repeat</t>
-        </is>
-      </c>
-      <c r="B156" t="inlineStr"/>
-      <c r="C156" t="inlineStr"/>
+          <t>select_one tipo_evid</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>evid_e1_tipo</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>Tipo de evidência</t>
+        </is>
+      </c>
       <c r="D156" t="inlineStr"/>
       <c r="E156" t="inlineStr"/>
       <c r="F156" t="inlineStr"/>
@@ -4694,14 +4722,26 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>end_group</t>
-        </is>
-      </c>
-      <c r="B157" t="inlineStr"/>
-      <c r="C157" t="inlineStr"/>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>evid_e1_tipo_outro</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>Especifique (Outro)</t>
+        </is>
+      </c>
       <c r="D157" t="inlineStr"/>
       <c r="E157" t="inlineStr"/>
-      <c r="F157" t="inlineStr"/>
+      <c r="F157" t="inlineStr">
+        <is>
+          <t>${evid_e1_tipo}='outro'</t>
+        </is>
+      </c>
       <c r="G157" t="inlineStr"/>
       <c r="H157" t="inlineStr"/>
       <c r="I157" t="inlineStr"/>
@@ -4710,18 +4750,102 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>end_group</t>
-        </is>
-      </c>
-      <c r="B158" t="inlineStr"/>
-      <c r="C158" t="inlineStr"/>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>evid_e1_desc</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>Descreva a evidência</t>
+        </is>
+      </c>
       <c r="D158" t="inlineStr"/>
       <c r="E158" t="inlineStr"/>
       <c r="F158" t="inlineStr"/>
-      <c r="G158" t="inlineStr"/>
+      <c r="G158" t="inlineStr">
+        <is>
+          <t>multiline</t>
+        </is>
+      </c>
       <c r="H158" t="inlineStr"/>
       <c r="I158" t="inlineStr"/>
       <c r="J158" t="inlineStr"/>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>file</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>evid_e1_anexo</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>Anexo (foto/documento) — opcional</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr"/>
+      <c r="E159" t="inlineStr"/>
+      <c r="F159" t="inlineStr"/>
+      <c r="G159" t="inlineStr"/>
+      <c r="H159" t="inlineStr"/>
+      <c r="I159" t="inlineStr"/>
+      <c r="J159" t="inlineStr"/>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>end_repeat</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr"/>
+      <c r="C160" t="inlineStr"/>
+      <c r="D160" t="inlineStr"/>
+      <c r="E160" t="inlineStr"/>
+      <c r="F160" t="inlineStr"/>
+      <c r="G160" t="inlineStr"/>
+      <c r="H160" t="inlineStr"/>
+      <c r="I160" t="inlineStr"/>
+      <c r="J160" t="inlineStr"/>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>end_group</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr"/>
+      <c r="C161" t="inlineStr"/>
+      <c r="D161" t="inlineStr"/>
+      <c r="E161" t="inlineStr"/>
+      <c r="F161" t="inlineStr"/>
+      <c r="G161" t="inlineStr"/>
+      <c r="H161" t="inlineStr"/>
+      <c r="I161" t="inlineStr"/>
+      <c r="J161" t="inlineStr"/>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>end_group</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr"/>
+      <c r="C162" t="inlineStr"/>
+      <c r="D162" t="inlineStr"/>
+      <c r="E162" t="inlineStr"/>
+      <c r="F162" t="inlineStr"/>
+      <c r="G162" t="inlineStr"/>
+      <c r="H162" t="inlineStr"/>
+      <c r="I162" t="inlineStr"/>
+      <c r="J162" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Adiciona confirmação final obrigatória aos formulários
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AahsCeqM2DTecRKsTTfJbG
</commit_message>
<xml_diff>
--- a/kobo/gestores_semana1_diagnostico.xlsx
+++ b/kobo/gestores_semana1_diagnostico.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J162"/>
+  <dimension ref="A1:J166"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4834,11 +4834,19 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>end_group</t>
-        </is>
-      </c>
-      <c r="B162" t="inlineStr"/>
-      <c r="C162" t="inlineStr"/>
+          <t>begin_group</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>confirmacao</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>Confirmação final</t>
+        </is>
+      </c>
       <c r="D162" t="inlineStr"/>
       <c r="E162" t="inlineStr"/>
       <c r="F162" t="inlineStr"/>
@@ -4846,6 +4854,90 @@
       <c r="H162" t="inlineStr"/>
       <c r="I162" t="inlineStr"/>
       <c r="J162" t="inlineStr"/>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>confirmacao_msg</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>Semana 1/5 concluída. Obrigado(a) pela sua participação! Suas respostas ajudam a construir um diagnóstico mais completo. Revise o que respondeu, confirme abaixo e clique em Enviar para concluir.</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr"/>
+      <c r="E163" t="inlineStr"/>
+      <c r="F163" t="inlineStr"/>
+      <c r="G163" t="inlineStr"/>
+      <c r="H163" t="inlineStr"/>
+      <c r="I163" t="inlineStr"/>
+      <c r="J163" t="inlineStr"/>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>select_one confirmo</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>confirmacao_envio</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>Revisei minhas respostas e confirmo o envio.</t>
+        </is>
+      </c>
+      <c r="D164" t="inlineStr"/>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="F164" t="inlineStr"/>
+      <c r="G164" t="inlineStr"/>
+      <c r="H164" t="inlineStr"/>
+      <c r="I164" t="inlineStr"/>
+      <c r="J164" t="inlineStr"/>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>end_group</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr"/>
+      <c r="C165" t="inlineStr"/>
+      <c r="D165" t="inlineStr"/>
+      <c r="E165" t="inlineStr"/>
+      <c r="F165" t="inlineStr"/>
+      <c r="G165" t="inlineStr"/>
+      <c r="H165" t="inlineStr"/>
+      <c r="I165" t="inlineStr"/>
+      <c r="J165" t="inlineStr"/>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>end_group</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr"/>
+      <c r="C166" t="inlineStr"/>
+      <c r="D166" t="inlineStr"/>
+      <c r="E166" t="inlineStr"/>
+      <c r="F166" t="inlineStr"/>
+      <c r="G166" t="inlineStr"/>
+      <c r="H166" t="inlineStr"/>
+      <c r="I166" t="inlineStr"/>
+      <c r="J166" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4858,7 +4950,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C185"/>
+  <dimension ref="A1:C186"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4881,17 +4973,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>concordo</t>
+          <t>confirmo</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>concordo</t>
+          <t>confirmo</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Sim, concordo em participar</t>
+          <t>Sim, confirmo o envio</t>
         </is>
       </c>
     </row>
@@ -4903,29 +4995,29 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>nao_concordo</t>
+          <t>concordo</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Não concordo</t>
+          <t>Sim, concordo em participar</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>sim_nao_ns</t>
+          <t>concordo</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>sim</t>
+          <t>nao_concordo</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Sim</t>
+          <t>Não concordo</t>
         </is>
       </c>
     </row>
@@ -4937,12 +5029,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>nao</t>
+          <t>sim</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim</t>
         </is>
       </c>
     </row>
@@ -4954,29 +5046,29 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>nao_sabemos</t>
+          <t>nao</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Não sabemos</t>
+          <t>Não</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>uf</t>
+          <t>sim_nao_ns</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>AC</t>
+          <t>nao_sabemos</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>AC</t>
+          <t>Não sabemos</t>
         </is>
       </c>
     </row>
@@ -4988,12 +5080,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>AL</t>
+          <t>AC</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>AL</t>
+          <t>AC</t>
         </is>
       </c>
     </row>
@@ -5005,12 +5097,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>AP</t>
+          <t>AL</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>AP</t>
+          <t>AL</t>
         </is>
       </c>
     </row>
@@ -5022,12 +5114,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>AM</t>
+          <t>AP</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>AM</t>
+          <t>AP</t>
         </is>
       </c>
     </row>
@@ -5039,12 +5131,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>BA</t>
+          <t>AM</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>BA</t>
+          <t>AM</t>
         </is>
       </c>
     </row>
@@ -5056,12 +5148,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>CE</t>
+          <t>BA</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>CE</t>
+          <t>BA</t>
         </is>
       </c>
     </row>
@@ -5073,12 +5165,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>DF</t>
+          <t>CE</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>DF</t>
+          <t>CE</t>
         </is>
       </c>
     </row>
@@ -5090,12 +5182,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>DF</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>DF</t>
         </is>
       </c>
     </row>
@@ -5107,12 +5199,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>GO</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>GO</t>
+          <t>ES</t>
         </is>
       </c>
     </row>
@@ -5124,12 +5216,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>GO</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>GO</t>
         </is>
       </c>
     </row>
@@ -5141,12 +5233,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>MT</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>MT</t>
+          <t>MA</t>
         </is>
       </c>
     </row>
@@ -5158,12 +5250,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>MS</t>
+          <t>MT</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>MS</t>
+          <t>MT</t>
         </is>
       </c>
     </row>
@@ -5175,12 +5267,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>MG</t>
+          <t>MS</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>MG</t>
+          <t>MS</t>
         </is>
       </c>
     </row>
@@ -5192,12 +5284,12 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>PA</t>
+          <t>MG</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>PA</t>
+          <t>MG</t>
         </is>
       </c>
     </row>
@@ -5209,12 +5301,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>PB</t>
+          <t>PA</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>PB</t>
+          <t>PA</t>
         </is>
       </c>
     </row>
@@ -5226,12 +5318,12 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>PR</t>
+          <t>PB</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>PR</t>
+          <t>PB</t>
         </is>
       </c>
     </row>
@@ -5243,12 +5335,12 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>PE</t>
+          <t>PR</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>PE</t>
+          <t>PR</t>
         </is>
       </c>
     </row>
@@ -5260,12 +5352,12 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>PE</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>PE</t>
         </is>
       </c>
     </row>
@@ -5277,12 +5369,12 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>RJ</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>RJ</t>
+          <t>PI</t>
         </is>
       </c>
     </row>
@@ -5294,12 +5386,12 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>RN</t>
+          <t>RJ</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>RN</t>
+          <t>RJ</t>
         </is>
       </c>
     </row>
@@ -5311,12 +5403,12 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>RS</t>
+          <t>RN</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>RS</t>
+          <t>RN</t>
         </is>
       </c>
     </row>
@@ -5328,12 +5420,12 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>RO</t>
+          <t>RS</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>RO</t>
+          <t>RS</t>
         </is>
       </c>
     </row>
@@ -5345,12 +5437,12 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>RR</t>
+          <t>RO</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>RR</t>
+          <t>RO</t>
         </is>
       </c>
     </row>
@@ -5362,12 +5454,12 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>SC</t>
+          <t>RR</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>SC</t>
+          <t>RR</t>
         </is>
       </c>
     </row>
@@ -5379,12 +5471,12 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>SP</t>
+          <t>SC</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>SP</t>
+          <t>SC</t>
         </is>
       </c>
     </row>
@@ -5396,12 +5488,12 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>SE</t>
+          <t>SP</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>SE</t>
+          <t>SP</t>
         </is>
       </c>
     </row>
@@ -5413,29 +5505,29 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>TO</t>
+          <t>SE</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>TO</t>
+          <t>SE</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>tipo_local</t>
+          <t>uf</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>escola</t>
+          <t>TO</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Escola</t>
+          <t>TO</t>
         </is>
       </c>
     </row>
@@ -5447,12 +5539,12 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>secretaria_municipal_de_educacao</t>
+          <t>escola</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Secretaria municipal de educação</t>
+          <t>Escola</t>
         </is>
       </c>
     </row>
@@ -5464,12 +5556,12 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>secretaria_estadual_de_educacao</t>
+          <t>secretaria_municipal_de_educacao</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Secretaria estadual de educação</t>
+          <t>Secretaria municipal de educação</t>
         </is>
       </c>
     </row>
@@ -5481,12 +5573,12 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>diretoria_coordenadoria_regional</t>
+          <t>secretaria_estadual_de_educacao</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Diretoria/coordenadoria regional de ensino</t>
+          <t>Secretaria estadual de educação</t>
         </is>
       </c>
     </row>
@@ -5498,29 +5590,29 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>outro</t>
+          <t>diretoria_coordenadoria_regional</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Outro</t>
+          <t>Diretoria/coordenadoria regional de ensino</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>rede</t>
+          <t>tipo_local</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>municipal</t>
+          <t>outro</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Municipal</t>
+          <t>Outro</t>
         </is>
       </c>
     </row>
@@ -5532,12 +5624,12 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>estadual</t>
+          <t>municipal</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Estadual</t>
+          <t>Municipal</t>
         </is>
       </c>
     </row>
@@ -5549,12 +5641,12 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>federal</t>
+          <t>estadual</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Federal</t>
+          <t>Estadual</t>
         </is>
       </c>
     </row>
@@ -5566,12 +5658,12 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>privado</t>
+          <t>federal</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Privado</t>
+          <t>Federal</t>
         </is>
       </c>
     </row>
@@ -5583,12 +5675,12 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>comunitario</t>
+          <t>privado</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Comunitário</t>
+          <t>Privado</t>
         </is>
       </c>
     </row>
@@ -5600,29 +5692,29 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>outro</t>
+          <t>comunitario</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Outro</t>
+          <t>Comunitário</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>localizacao</t>
+          <t>rede</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>urbana</t>
+          <t>outro</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Urbana</t>
+          <t>Outro</t>
         </is>
       </c>
     </row>
@@ -5634,12 +5726,12 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>rural</t>
+          <t>urbana</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Urbana</t>
         </is>
       </c>
     </row>
@@ -5651,12 +5743,12 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>periurbana_de_transicao</t>
+          <t>rural</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Periurbana / de transição</t>
+          <t>Rural</t>
         </is>
       </c>
     </row>
@@ -5668,29 +5760,29 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>nao_sabe</t>
+          <t>periurbana_de_transicao</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Não sabe</t>
+          <t>Periurbana / de transição</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>contextos</t>
+          <t>localizacao</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>educacao_do_campo</t>
+          <t>nao_sabe</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Educação do Campo</t>
+          <t>Não sabe</t>
         </is>
       </c>
     </row>
@@ -5702,12 +5794,12 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>territorio_indigena</t>
+          <t>educacao_do_campo</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Território indígena</t>
+          <t>Educação do Campo</t>
         </is>
       </c>
     </row>
@@ -5719,12 +5811,12 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>quilombola</t>
+          <t>territorio_indigena</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Quilombola</t>
+          <t>Território indígena</t>
         </is>
       </c>
     </row>
@@ -5736,12 +5828,12 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>ribeirinho</t>
+          <t>quilombola</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Ribeirinho</t>
+          <t>Quilombola</t>
         </is>
       </c>
     </row>
@@ -5753,12 +5845,12 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>caicara</t>
+          <t>ribeirinho</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Caiçara</t>
+          <t>Ribeirinho</t>
         </is>
       </c>
     </row>
@@ -5770,12 +5862,12 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>extrativista</t>
+          <t>caicara</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Extrativista</t>
+          <t>Caiçara</t>
         </is>
       </c>
     </row>
@@ -5787,12 +5879,12 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>assentamento</t>
+          <t>extrativista</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Assentamento</t>
+          <t>Extrativista</t>
         </is>
       </c>
     </row>
@@ -5804,12 +5896,12 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>outro</t>
+          <t>assentamento</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Outro</t>
+          <t>Assentamento</t>
         </is>
       </c>
     </row>
@@ -5821,12 +5913,12 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>nenhum</t>
+          <t>outro</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Nenhum</t>
+          <t>Outro</t>
         </is>
       </c>
     </row>
@@ -5838,29 +5930,29 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>nao_sabe</t>
+          <t>nenhum</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Não sabe</t>
+          <t>Nenhum</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>funcao</t>
+          <t>contextos</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>diretor</t>
+          <t>nao_sabe</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Diretor(a)</t>
+          <t>Não sabe</t>
         </is>
       </c>
     </row>
@@ -5872,12 +5964,12 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>vice_diretor</t>
+          <t>diretor</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Vice-diretor(a)</t>
+          <t>Diretor(a)</t>
         </is>
       </c>
     </row>
@@ -5889,12 +5981,12 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>coordenador_pedagogico</t>
+          <t>vice_diretor</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Coordenador(a) pedagógico(a)</t>
+          <t>Vice-diretor(a)</t>
         </is>
       </c>
     </row>
@@ -5906,12 +5998,12 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>supervisor_pedagogico</t>
+          <t>coordenador_pedagogico</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Supervisor(a) pedagógico(a)</t>
+          <t>Coordenador(a) pedagógico(a)</t>
         </is>
       </c>
     </row>
@@ -5923,12 +6015,12 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>orientador_educacional</t>
+          <t>supervisor_pedagogico</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Orientador(a) educacional</t>
+          <t>Supervisor(a) pedagógico(a)</t>
         </is>
       </c>
     </row>
@@ -5940,12 +6032,12 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>secretario_escolar</t>
+          <t>orientador_educacional</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Secretário(a) escolar</t>
+          <t>Orientador(a) educacional</t>
         </is>
       </c>
     </row>
@@ -5957,29 +6049,29 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>outro</t>
+          <t>secretario_escolar</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Outro (equipe gestora)</t>
+          <t>Secretário(a) escolar</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>formacao</t>
+          <t>funcao</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>ensino_fundamental</t>
+          <t>outro</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Ensino Fundamental</t>
+          <t>Outro (equipe gestora)</t>
         </is>
       </c>
     </row>
@@ -5991,12 +6083,12 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>ensino_medio_magisterio</t>
+          <t>ensino_fundamental</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Ensino Médio / Magistério</t>
+          <t>Ensino Fundamental</t>
         </is>
       </c>
     </row>
@@ -6008,12 +6100,12 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>graduacao</t>
+          <t>ensino_medio_magisterio</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Graduação</t>
+          <t>Ensino Médio / Magistério</t>
         </is>
       </c>
     </row>
@@ -6025,12 +6117,12 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>pos_graduacao</t>
+          <t>graduacao</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Pós-graduação (especialização)</t>
+          <t>Graduação</t>
         </is>
       </c>
     </row>
@@ -6042,12 +6134,12 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>mestrado</t>
+          <t>pos_graduacao</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Mestrado</t>
+          <t>Pós-graduação (especialização)</t>
         </is>
       </c>
     </row>
@@ -6059,12 +6151,12 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>doutorado</t>
+          <t>mestrado</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Doutorado</t>
+          <t>Mestrado</t>
         </is>
       </c>
     </row>
@@ -6076,29 +6168,29 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>nao_sabe_nao_se_aplica</t>
+          <t>doutorado</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Não sabe / não se aplica</t>
+          <t>Doutorado</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>estado_infra</t>
+          <t>formacao</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>inexistente</t>
+          <t>nao_sabe_nao_se_aplica</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Inexistente</t>
+          <t>Não sabe / não se aplica</t>
         </is>
       </c>
     </row>
@@ -6110,12 +6202,12 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>inadequado</t>
+          <t>inexistente</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Inadequado</t>
+          <t>Inexistente</t>
         </is>
       </c>
     </row>
@@ -6127,12 +6219,12 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>regular</t>
+          <t>inadequado</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Regular</t>
+          <t>Inadequado</t>
         </is>
       </c>
     </row>
@@ -6144,12 +6236,12 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>bom</t>
+          <t>regular</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Bom</t>
+          <t>Regular</t>
         </is>
       </c>
     </row>
@@ -6161,12 +6253,12 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>nao_se_aplica</t>
+          <t>bom</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Não se aplica</t>
+          <t>Bom</t>
         </is>
       </c>
     </row>
@@ -6178,29 +6270,29 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>nao_sabe</t>
+          <t>nao_se_aplica</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Não sabe</t>
+          <t>Não se aplica</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>qtd_rede</t>
+          <t>estado_infra</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>em_nenhuma</t>
+          <t>nao_sabe</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Em nenhuma</t>
+          <t>Não sabe</t>
         </is>
       </c>
     </row>
@@ -6212,12 +6304,12 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>em_poucas</t>
+          <t>em_nenhuma</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Em poucas</t>
+          <t>Em nenhuma</t>
         </is>
       </c>
     </row>
@@ -6229,12 +6321,12 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>em_cerca_de_metade</t>
+          <t>em_poucas</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Em cerca de metade</t>
+          <t>Em poucas</t>
         </is>
       </c>
     </row>
@@ -6246,12 +6338,12 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>na_maioria</t>
+          <t>em_cerca_de_metade</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Na maioria</t>
+          <t>Em cerca de metade</t>
         </is>
       </c>
     </row>
@@ -6263,12 +6355,12 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>em_todas</t>
+          <t>na_maioria</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Em todas</t>
+          <t>Na maioria</t>
         </is>
       </c>
     </row>
@@ -6280,29 +6372,29 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>nao_sabe</t>
+          <t>em_todas</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Não sabe</t>
+          <t>Em todas</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>qtd_rede_tab</t>
+          <t>qtd_rede</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>em_nenhuma</t>
+          <t>nao_sabe</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Em nenhuma</t>
+          <t>Não sabe</t>
         </is>
       </c>
     </row>
@@ -6314,12 +6406,12 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>em_poucas</t>
+          <t>em_nenhuma</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Em poucas</t>
+          <t>Em nenhuma</t>
         </is>
       </c>
     </row>
@@ -6331,12 +6423,12 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>em_cerca_de_metade</t>
+          <t>em_poucas</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Em cerca de metade</t>
+          <t>Em poucas</t>
         </is>
       </c>
     </row>
@@ -6348,12 +6440,12 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>na_maioria</t>
+          <t>em_cerca_de_metade</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Na maioria</t>
+          <t>Em cerca de metade</t>
         </is>
       </c>
     </row>
@@ -6365,12 +6457,12 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>em_todas</t>
+          <t>na_maioria</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Em todas</t>
+          <t>Na maioria</t>
         </is>
       </c>
     </row>
@@ -6382,12 +6474,12 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>nao_se_aplica</t>
+          <t>em_todas</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Não se aplica</t>
+          <t>Em todas</t>
         </is>
       </c>
     </row>
@@ -6399,29 +6491,29 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>nao_sabe</t>
+          <t>nao_se_aplica</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Não sabe</t>
+          <t>Não se aplica</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>termica</t>
+          <t>qtd_rede_tab</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>muito_quente_no_verao</t>
+          <t>nao_sabe</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Muito quente no verão</t>
+          <t>Não sabe</t>
         </is>
       </c>
     </row>
@@ -6433,12 +6525,12 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>muito_fria_no_inverno</t>
+          <t>muito_quente_no_verao</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Muito fria no inverno</t>
+          <t>Muito quente no verão</t>
         </is>
       </c>
     </row>
@@ -6450,12 +6542,12 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>adequada_na_maior_parte_do_ano</t>
+          <t>muito_fria_no_inverno</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Adequada na maior parte do ano</t>
+          <t>Muito fria no inverno</t>
         </is>
       </c>
     </row>
@@ -6467,12 +6559,12 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>muito_variavel_sem_padrao_sazona</t>
+          <t>adequada_na_maior_parte_do_ano</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Muito variável, sem padrão sazonal claro</t>
+          <t>Adequada na maior parte do ano</t>
         </is>
       </c>
     </row>
@@ -6484,29 +6576,29 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>nao_sabe</t>
+          <t>muito_variavel_sem_padrao_sazona</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Não sabe</t>
+          <t>Muito variável, sem padrão sazonal claro</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>prob_estrut</t>
+          <t>termica</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>mofo</t>
+          <t>nao_sabe</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Mofo</t>
+          <t>Não sabe</t>
         </is>
       </c>
     </row>
@@ -6518,12 +6610,12 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>infiltracao</t>
+          <t>mofo</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Infiltração</t>
+          <t>Mofo</t>
         </is>
       </c>
     </row>
@@ -6535,12 +6627,12 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>calor_excessivo</t>
+          <t>infiltracao</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Calor excessivo</t>
+          <t>Infiltração</t>
         </is>
       </c>
     </row>
@@ -6552,12 +6644,12 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>frio_excessivo</t>
+          <t>calor_excessivo</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Frio excessivo</t>
+          <t>Calor excessivo</t>
         </is>
       </c>
     </row>
@@ -6569,12 +6661,12 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>falta_de_ventilacao</t>
+          <t>frio_excessivo</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Falta de ventilação</t>
+          <t>Frio excessivo</t>
         </is>
       </c>
     </row>
@@ -6586,29 +6678,29 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>outro</t>
+          <t>falta_de_ventilacao</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Outro</t>
+          <t>Falta de ventilação</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>agua_fonte</t>
+          <t>prob_estrut</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>rede_publica</t>
+          <t>outro</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Rede pública</t>
+          <t>Outro</t>
         </is>
       </c>
     </row>
@@ -6620,12 +6712,12 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>poco</t>
+          <t>rede_publica</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Poço</t>
+          <t>Rede pública</t>
         </is>
       </c>
     </row>
@@ -6637,12 +6729,12 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>nascente</t>
+          <t>poco</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Nascente</t>
+          <t>Poço</t>
         </is>
       </c>
     </row>
@@ -6654,12 +6746,12 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>cisterna</t>
+          <t>nascente</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Cisterna</t>
+          <t>Nascente</t>
         </is>
       </c>
     </row>
@@ -6671,12 +6763,12 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>outro</t>
+          <t>cisterna</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Outra</t>
+          <t>Cisterna</t>
         </is>
       </c>
     </row>
@@ -6688,29 +6780,29 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>nao_sabe</t>
+          <t>outro</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Não sabe</t>
+          <t>Outra</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>infra_hidrica</t>
+          <t>agua_fonte</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>reservatorio_caixa_d_agua</t>
+          <t>nao_sabe</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Reservatório / caixa d'água</t>
+          <t>Não sabe</t>
         </is>
       </c>
     </row>
@@ -6722,12 +6814,12 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>filtro_purificador</t>
+          <t>reservatorio_caixa_d_agua</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>Filtro / purificador</t>
+          <t>Reservatório / caixa d'água</t>
         </is>
       </c>
     </row>
@@ -6739,12 +6831,12 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>bebedouros</t>
+          <t>filtro_purificador</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Bebedouros</t>
+          <t>Filtro / purificador</t>
         </is>
       </c>
     </row>
@@ -6756,12 +6848,12 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>rede_encanada_interna</t>
+          <t>bebedouros</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>Rede encanada interna</t>
+          <t>Bebedouros</t>
         </is>
       </c>
     </row>
@@ -6773,12 +6865,12 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>outro</t>
+          <t>rede_encanada_interna</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Outro</t>
+          <t>Rede encanada interna</t>
         </is>
       </c>
     </row>
@@ -6790,29 +6882,29 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>nao_sabe</t>
+          <t>outro</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>Não sabe</t>
+          <t>Outro</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>esgoto</t>
+          <t>infra_hidrica</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>rede_coletora</t>
+          <t>nao_sabe</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>Rede coletora</t>
+          <t>Não sabe</t>
         </is>
       </c>
     </row>
@@ -6824,12 +6916,12 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>fossa_septica</t>
+          <t>rede_coletora</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>Fossa séptica</t>
+          <t>Rede coletora</t>
         </is>
       </c>
     </row>
@@ -6841,12 +6933,12 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>fossa_rudimentar</t>
+          <t>fossa_septica</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>Fossa rudimentar</t>
+          <t>Fossa séptica</t>
         </is>
       </c>
     </row>
@@ -6858,12 +6950,12 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>ceu_aberto</t>
+          <t>fossa_rudimentar</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>Céu aberto</t>
+          <t>Fossa rudimentar</t>
         </is>
       </c>
     </row>
@@ -6875,12 +6967,12 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>outro</t>
+          <t>ceu_aberto</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>Outro</t>
+          <t>Céu aberto</t>
         </is>
       </c>
     </row>
@@ -6892,29 +6984,29 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>nao_sabe</t>
+          <t>outro</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>Não sabe</t>
+          <t>Outro</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>impacto_alag</t>
+          <t>esgoto</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>interrupcao_de_aulas</t>
+          <t>nao_sabe</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>Interrupção de aulas</t>
+          <t>Não sabe</t>
         </is>
       </c>
     </row>
@@ -6926,12 +7018,12 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>danos_a_estrutura</t>
+          <t>interrupcao_de_aulas</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>Danos à estrutura</t>
+          <t>Interrupção de aulas</t>
         </is>
       </c>
     </row>
@@ -6943,12 +7035,12 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>acesso_interrompido</t>
+          <t>danos_a_estrutura</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>Dificuldade ou interrupção do acesso ao local</t>
+          <t>Danos à estrutura</t>
         </is>
       </c>
     </row>
@@ -6960,12 +7052,12 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>baixa_adesao</t>
+          <t>acesso_interrompido</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>Baixa adesão dos estudantes (aulas mantidas, mas poucos conseguem frequentar)</t>
+          <t>Dificuldade ou interrupção do acesso ao local</t>
         </is>
       </c>
     </row>
@@ -6977,29 +7069,29 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>outro</t>
+          <t>baixa_adesao</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>Outro</t>
+          <t>Baixa adesão dos estudantes (aulas mantidas, mas poucos conseguem frequentar)</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>destino_res</t>
+          <t>impacto_alag</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>coleta_publica</t>
+          <t>outro</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>Coleta pública</t>
+          <t>Outro</t>
         </is>
       </c>
     </row>
@@ -7011,12 +7103,12 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>coleta_seletiva</t>
+          <t>coleta_publica</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>Coleta seletiva</t>
+          <t>Coleta pública</t>
         </is>
       </c>
     </row>
@@ -7028,12 +7120,12 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>cooperativa</t>
+          <t>coleta_seletiva</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>Cooperativa</t>
+          <t>Coleta seletiva</t>
         </is>
       </c>
     </row>
@@ -7045,12 +7137,12 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>compostagem</t>
+          <t>cooperativa</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>Compostagem</t>
+          <t>Cooperativa</t>
         </is>
       </c>
     </row>
@@ -7062,12 +7154,12 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>reutilizacao</t>
+          <t>compostagem</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>Reutilização</t>
+          <t>Compostagem</t>
         </is>
       </c>
     </row>
@@ -7079,12 +7171,12 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>queima</t>
+          <t>reutilizacao</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>Queima</t>
+          <t>Reutilização</t>
         </is>
       </c>
     </row>
@@ -7096,12 +7188,12 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>enterramento</t>
+          <t>queima</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>Enterramento</t>
+          <t>Queima</t>
         </is>
       </c>
     </row>
@@ -7113,12 +7205,12 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>outro</t>
+          <t>enterramento</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>Outro</t>
+          <t>Enterramento</t>
         </is>
       </c>
     </row>
@@ -7130,29 +7222,29 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>nao_sabe</t>
+          <t>outro</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>Não sabe</t>
+          <t>Outro</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>prob_res</t>
+          <t>destino_res</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>aterro_sanitario</t>
+          <t>nao_sabe</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>Aterro sanitário</t>
+          <t>Não sabe</t>
         </is>
       </c>
     </row>
@@ -7164,12 +7256,12 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>lixao</t>
+          <t>aterro_sanitario</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>Lixão</t>
+          <t>Aterro sanitário</t>
         </is>
       </c>
     </row>
@@ -7181,12 +7273,12 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>queima_de_residuos</t>
+          <t>lixao</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>Queima de resíduos</t>
+          <t>Lixão</t>
         </is>
       </c>
     </row>
@@ -7198,12 +7290,12 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>acumulo_de_residuos_no_entorno</t>
+          <t>queima_de_residuos</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>Acúmulo de resíduos no entorno</t>
+          <t>Queima de resíduos</t>
         </is>
       </c>
     </row>
@@ -7215,12 +7307,12 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>outro</t>
+          <t>acumulo_de_residuos_no_entorno</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>Outro</t>
+          <t>Acúmulo de resíduos no entorno</t>
         </is>
       </c>
     </row>
@@ -7232,12 +7324,12 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>nenhum</t>
+          <t>outro</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>Nenhum</t>
+          <t>Outro</t>
         </is>
       </c>
     </row>
@@ -7249,29 +7341,29 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>nao_sabe</t>
+          <t>nenhum</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>Não sabe</t>
+          <t>Nenhum</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>elementos</t>
+          <t>prob_res</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>rios_corregos</t>
+          <t>nao_sabe</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>Rios/córregos</t>
+          <t>Não sabe</t>
         </is>
       </c>
     </row>
@@ -7283,12 +7375,12 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>lagoas_lagos_reservatorios</t>
+          <t>rios_corregos</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>Lagoas/lagos/reservatórios</t>
+          <t>Rios/córregos</t>
         </is>
       </c>
     </row>
@@ -7300,12 +7392,12 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>areas_de_vegetacao_nativa</t>
+          <t>lagoas_lagos_reservatorios</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>Áreas de vegetação nativa (matas, florestas, campos)</t>
+          <t>Lagoas/lagos/reservatórios</t>
         </is>
       </c>
     </row>
@@ -7317,12 +7409,12 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>parques</t>
+          <t>areas_de_vegetacao_nativa</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>Parques</t>
+          <t>Áreas de vegetação nativa (matas, florestas, campos)</t>
         </is>
       </c>
     </row>
@@ -7334,12 +7426,12 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>encostas</t>
+          <t>parques</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>Encostas</t>
+          <t>Parques</t>
         </is>
       </c>
     </row>
@@ -7351,12 +7443,12 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>agricultura</t>
+          <t>encostas</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>Agricultura</t>
+          <t>Encostas</t>
         </is>
       </c>
     </row>
@@ -7368,12 +7460,12 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>industria</t>
+          <t>agricultura</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>Indústria</t>
+          <t>Agricultura</t>
         </is>
       </c>
     </row>
@@ -7385,12 +7477,12 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>mineracao</t>
+          <t>industria</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>Mineração</t>
+          <t>Indústria</t>
         </is>
       </c>
     </row>
@@ -7402,12 +7494,12 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>aterro_lixao</t>
+          <t>mineracao</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>Aterro/lixão</t>
+          <t>Mineração</t>
         </is>
       </c>
     </row>
@@ -7419,12 +7511,12 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>areas_queimadas</t>
+          <t>aterro_lixao</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>Áreas queimadas</t>
+          <t>Aterro/lixão</t>
         </is>
       </c>
     </row>
@@ -7436,12 +7528,12 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>areas_inundaveis</t>
+          <t>areas_queimadas</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>Áreas inundáveis</t>
+          <t>Áreas queimadas</t>
         </is>
       </c>
     </row>
@@ -7453,12 +7545,12 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>comercios</t>
+          <t>areas_inundaveis</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>Comércios</t>
+          <t>Áreas inundáveis</t>
         </is>
       </c>
     </row>
@@ -7470,12 +7562,12 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>outras_areas_degradadas</t>
+          <t>comercios</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>Outras áreas degradadas</t>
+          <t>Comércios</t>
         </is>
       </c>
     </row>
@@ -7487,12 +7579,12 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>equipamentos_urbanos</t>
+          <t>outras_areas_degradadas</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>Equipamentos Urbanos</t>
+          <t>Outras áreas degradadas</t>
         </is>
       </c>
     </row>
@@ -7504,29 +7596,29 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>outro</t>
+          <t>equipamentos_urbanos</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>Outros</t>
+          <t>Equipamentos Urbanos</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>relacao_elem</t>
+          <t>elementos</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>ambiente</t>
+          <t>outro</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>Ambiente</t>
+          <t>Outros</t>
         </is>
       </c>
     </row>
@@ -7538,12 +7630,12 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>cultura</t>
+          <t>ambiente</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>Cultura</t>
+          <t>Ambiente</t>
         </is>
       </c>
     </row>
@@ -7555,12 +7647,12 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>uso_comunitario</t>
+          <t>cultura</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>Uso comunitário</t>
+          <t>Cultura</t>
         </is>
       </c>
     </row>
@@ -7572,12 +7664,12 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>renda</t>
+          <t>uso_comunitario</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>Renda</t>
+          <t>Uso comunitário</t>
         </is>
       </c>
     </row>
@@ -7589,12 +7681,12 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>risco</t>
+          <t>renda</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>Risco</t>
+          <t>Renda</t>
         </is>
       </c>
     </row>
@@ -7606,12 +7698,12 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>degradacao</t>
+          <t>risco</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>Degradação</t>
+          <t>Risco</t>
         </is>
       </c>
     </row>
@@ -7623,12 +7715,12 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>conflito</t>
+          <t>degradacao</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>Conflito</t>
+          <t>Degradação</t>
         </is>
       </c>
     </row>
@@ -7640,12 +7732,12 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>outro</t>
+          <t>conflito</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>Outra</t>
+          <t>Conflito</t>
         </is>
       </c>
     </row>
@@ -7657,29 +7749,29 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>nao_sabe</t>
+          <t>outro</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>Não sabe</t>
+          <t>Outra</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>ativ_econ</t>
+          <t>relacao_elem</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>agricultura</t>
+          <t>nao_sabe</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>Agricultura</t>
+          <t>Não sabe</t>
         </is>
       </c>
     </row>
@@ -7691,12 +7783,12 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>pecuaria</t>
+          <t>agricultura</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>Pecuária</t>
+          <t>Agricultura</t>
         </is>
       </c>
     </row>
@@ -7708,12 +7800,12 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>comercio</t>
+          <t>pecuaria</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>Comércio</t>
+          <t>Pecuária</t>
         </is>
       </c>
     </row>
@@ -7725,12 +7817,12 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>industria</t>
+          <t>comercio</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>Indústria</t>
+          <t>Comércio</t>
         </is>
       </c>
     </row>
@@ -7742,12 +7834,12 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>turismo</t>
+          <t>industria</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>Turismo</t>
+          <t>Indústria</t>
         </is>
       </c>
     </row>
@@ -7759,12 +7851,12 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>pesca</t>
+          <t>turismo</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>Pesca</t>
+          <t>Turismo</t>
         </is>
       </c>
     </row>
@@ -7776,12 +7868,12 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>extrativismo</t>
+          <t>pesca</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>Extrativismo</t>
+          <t>Pesca</t>
         </is>
       </c>
     </row>
@@ -7793,29 +7885,29 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>outro</t>
+          <t>extrativismo</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>Outro</t>
+          <t>Extrativismo</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>impacto_clima</t>
+          <t>ativ_econ</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>interrupcao_de_aulas</t>
+          <t>outro</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>Interrupção de aulas</t>
+          <t>Outro</t>
         </is>
       </c>
     </row>
@@ -7827,12 +7919,12 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>danos_materiais</t>
+          <t>interrupcao_de_aulas</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>Danos materiais</t>
+          <t>Interrupção de aulas</t>
         </is>
       </c>
     </row>
@@ -7844,12 +7936,12 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>deslocamento_de_pessoas</t>
+          <t>danos_materiais</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>Deslocamento de pessoas (necessidade de migração)</t>
+          <t>Danos materiais</t>
         </is>
       </c>
     </row>
@@ -7861,12 +7953,12 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>perdas</t>
+          <t>deslocamento_de_pessoas</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>Óbitos</t>
+          <t>Deslocamento de pessoas (necessidade de migração)</t>
         </is>
       </c>
     </row>
@@ -7878,12 +7970,12 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>impacto_emocional</t>
+          <t>perdas</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>Impacto emocional</t>
+          <t>Óbitos</t>
         </is>
       </c>
     </row>
@@ -7895,29 +7987,29 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>outro</t>
+          <t>impacto_emocional</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>Outro</t>
+          <t>Impacto emocional</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>tipo_evid</t>
+          <t>impacto_clima</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>observacao_direta</t>
+          <t>outro</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>Observação direta</t>
+          <t>Outro</t>
         </is>
       </c>
     </row>
@@ -7929,12 +8021,12 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>documento</t>
+          <t>observacao_direta</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>Documento</t>
+          <t>Observação direta</t>
         </is>
       </c>
     </row>
@@ -7946,12 +8038,12 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>foto</t>
+          <t>documento</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>Foto</t>
+          <t>Documento</t>
         </is>
       </c>
     </row>
@@ -7963,12 +8055,12 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>depoimento</t>
+          <t>foto</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>Depoimento</t>
+          <t>Foto</t>
         </is>
       </c>
     </row>
@@ -7980,12 +8072,12 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>registro_historico</t>
+          <t>depoimento</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>Registro histórico</t>
+          <t>Depoimento</t>
         </is>
       </c>
     </row>
@@ -7997,10 +8089,27 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
+          <t>registro_historico</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>Registro histórico</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>tipo_evid</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
           <t>outro</t>
         </is>
       </c>
-      <c r="C185" t="inlineStr">
+      <c r="C186" t="inlineStr">
         <is>
           <t>Outra</t>
         </is>

</xml_diff>